<commit_message>
📅 日报更新 2026-08-16 14:03
</commit_message>
<xml_diff>
--- a/data/exports/王颖瑜伽/dist_order_2026-08-16.xlsx
+++ b/data/exports/王颖瑜伽/dist_order_2026-08-16.xlsx
@@ -125,11 +125,11 @@
     </row>
     <row r="2" spans="1:14">
       <c r="A2" s="0">
-        <v>49197594</v>
+        <v>49297749</v>
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>李秀燕健康顾问</t>
+          <t>沈雨凤</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
@@ -154,7 +154,7 @@
       </c>
       <c r="G2" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:55:55</t>
+          <t>2026-08-16 21:27:24</t>
         </is>
       </c>
       <c r="H2" s="0" t="inlineStr">
@@ -184,17 +184,17 @@
       </c>
       <c r="M2" s="0" t="inlineStr">
         <is>
-          <t>4500000383202608135550322726</t>
+          <t>4500000375202608164415130639</t>
         </is>
       </c>
     </row>
     <row r="3" spans="1:14">
       <c r="A3" s="0">
-        <v>49197555</v>
+        <v>49297736</v>
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t>FXH*</t>
+          <t>莉莉</t>
         </is>
       </c>
       <c r="C3" s="0" t="inlineStr">
@@ -219,7 +219,7 @@
       </c>
       <c r="G3" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:55:10</t>
+          <t>2026-08-16 21:27:09</t>
         </is>
       </c>
       <c r="H3" s="0" t="inlineStr">
@@ -249,17 +249,17 @@
       </c>
       <c r="M3" s="0" t="inlineStr">
         <is>
-          <t>4500000376202608139667116905</t>
+          <t>4500000369202608163428098661</t>
         </is>
       </c>
     </row>
     <row r="4" spans="1:14">
       <c r="A4" s="0">
-        <v>49197551</v>
+        <v>49297679</v>
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>书英</t>
+          <t>孔平</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
@@ -284,7 +284,7 @@
       </c>
       <c r="G4" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:55:09</t>
+          <t>2026-08-16 21:25:57</t>
         </is>
       </c>
       <c r="H4" s="0" t="inlineStr">
@@ -314,17 +314,17 @@
       </c>
       <c r="M4" s="0" t="inlineStr">
         <is>
-          <t>4500000363202608135183726220</t>
+          <t>4500000367202608165709204884</t>
         </is>
       </c>
     </row>
     <row r="5" spans="1:14">
       <c r="A5" s="0">
-        <v>49197500</v>
+        <v>49296893</v>
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t>求智慧</t>
+          <t>逍遥仙子</t>
         </is>
       </c>
       <c r="C5" s="0" t="inlineStr">
@@ -349,7 +349,7 @@
       </c>
       <c r="G5" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:54:20</t>
+          <t>2026-08-16 21:04:30</t>
         </is>
       </c>
       <c r="H5" s="0" t="inlineStr">
@@ -379,17 +379,17 @@
       </c>
       <c r="M5" s="0" t="inlineStr">
         <is>
-          <t>4500000356202608136477567012</t>
+          <t>4500000316202608167690459739</t>
         </is>
       </c>
     </row>
     <row r="6" spans="1:14">
       <c r="A6" s="0">
-        <v>49196660</v>
+        <v>49296884</v>
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t>陈书先</t>
+          <t>百佳惠大瑞丰药房曹利红</t>
         </is>
       </c>
       <c r="C6" s="0" t="inlineStr">
@@ -414,7 +414,7 @@
       </c>
       <c r="G6" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:35:55</t>
+          <t>2026-08-16 21:04:16</t>
         </is>
       </c>
       <c r="H6" s="0" t="inlineStr">
@@ -444,17 +444,17 @@
       </c>
       <c r="M6" s="0" t="inlineStr">
         <is>
-          <t>4500000362202608137513582005</t>
+          <t>4500000332202608162032983613</t>
         </is>
       </c>
     </row>
     <row r="7" spans="1:14">
       <c r="A7" s="0">
-        <v>49196649</v>
+        <v>49296864</v>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>chenchen</t>
+          <t>曹景玉</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
@@ -479,7 +479,7 @@
       </c>
       <c r="G7" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:35:37</t>
+          <t>2026-08-16 21:03:45</t>
         </is>
       </c>
       <c r="H7" s="0" t="inlineStr">
@@ -509,17 +509,17 @@
       </c>
       <c r="M7" s="0" t="inlineStr">
         <is>
-          <t>4500000360202608131193472561</t>
+          <t>4500000331202608163779658463</t>
         </is>
       </c>
     </row>
     <row r="8" spans="1:14">
       <c r="A8" s="0">
-        <v>49196616</v>
+        <v>49296863</v>
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>因子</t>
+          <t>石陆萍</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
@@ -544,7 +544,7 @@
       </c>
       <c r="G8" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:35:34</t>
+          <t>2026-08-16 21:04:13</t>
         </is>
       </c>
       <c r="H8" s="0" t="inlineStr">
@@ -574,17 +574,17 @@
       </c>
       <c r="M8" s="0" t="inlineStr">
         <is>
-          <t>4500000381202608131084069069</t>
+          <t>4500000351202608161473678444</t>
         </is>
       </c>
     </row>
     <row r="9" spans="1:14">
       <c r="A9" s="0">
-        <v>49196580</v>
+        <v>49296849</v>
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t>包容</t>
+          <t>阿荣</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
@@ -609,7 +609,7 @@
       </c>
       <c r="G9" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:34:49</t>
+          <t>2026-08-16 21:03:43</t>
         </is>
       </c>
       <c r="H9" s="0" t="inlineStr">
@@ -639,17 +639,17 @@
       </c>
       <c r="M9" s="0" t="inlineStr">
         <is>
-          <t>4500000329202608134515206220</t>
+          <t>4500000318202608169868333535</t>
         </is>
       </c>
     </row>
     <row r="10" spans="1:14">
       <c r="A10" s="0">
-        <v>49196556</v>
+        <v>49296823</v>
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t>小芳</t>
+          <t>周少丽</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
@@ -674,7 +674,7 @@
       </c>
       <c r="G10" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:34:00</t>
+          <t>2026-08-16 21:03:17</t>
         </is>
       </c>
       <c r="H10" s="0" t="inlineStr">
@@ -704,17 +704,17 @@
       </c>
       <c r="M10" s="0" t="inlineStr">
         <is>
-          <t>4500000380202608131586040016</t>
+          <t>4500000315202608169179019788</t>
         </is>
       </c>
     </row>
     <row r="11" spans="1:14">
       <c r="A11" s="0">
-        <v>49196547</v>
+        <v>49296822</v>
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t>雷宁</t>
+          <t>雨花石</t>
         </is>
       </c>
       <c r="C11" s="0" t="inlineStr">
@@ -739,7 +739,7 @@
       </c>
       <c r="G11" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:34:30</t>
+          <t>2026-08-16 21:03:16</t>
         </is>
       </c>
       <c r="H11" s="0" t="inlineStr">
@@ -769,17 +769,17 @@
       </c>
       <c r="M11" s="0" t="inlineStr">
         <is>
-          <t>4500000368202608133116145497</t>
+          <t>4500000367202608166345332381</t>
         </is>
       </c>
     </row>
     <row r="12" spans="1:14">
       <c r="A12" s="0">
-        <v>49196546</v>
+        <v>49293860</v>
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t>兰莓</t>
+          <t>树玲</t>
         </is>
       </c>
       <c r="C12" s="0" t="inlineStr">
@@ -804,7 +804,7 @@
       </c>
       <c r="G12" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:56:17</t>
+          <t>2026-08-16 19:55:26</t>
         </is>
       </c>
       <c r="H12" s="0" t="inlineStr">
@@ -834,17 +834,17 @@
       </c>
       <c r="M12" s="0" t="inlineStr">
         <is>
-          <t>4500000352202608136989637138</t>
+          <t>4500000342202608168589310428</t>
         </is>
       </c>
     </row>
     <row r="13" spans="1:14">
       <c r="A13" s="0">
-        <v>49196528</v>
+        <v>49293858</v>
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t>赵子睿奶奶</t>
+          <t>芬芳</t>
         </is>
       </c>
       <c r="C13" s="0" t="inlineStr">
@@ -869,7 +869,7 @@
       </c>
       <c r="G13" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:33:22</t>
+          <t>2026-08-16 19:55:42</t>
         </is>
       </c>
       <c r="H13" s="0" t="inlineStr">
@@ -899,17 +899,17 @@
       </c>
       <c r="M13" s="0" t="inlineStr">
         <is>
-          <t>4500000345202608137236789446</t>
+          <t>4500000358202608162910375128</t>
         </is>
       </c>
     </row>
     <row r="14" spans="1:14">
       <c r="A14" s="0">
-        <v>49196510</v>
+        <v>49197594</v>
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>山岭巨人</t>
+          <t>李秀燕健康顾问</t>
         </is>
       </c>
       <c r="C14" s="0" t="inlineStr">
@@ -934,7 +934,7 @@
       </c>
       <c r="G14" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:35:22</t>
+          <t>2026-08-13 21:55:55</t>
         </is>
       </c>
       <c r="H14" s="0" t="inlineStr">
@@ -964,17 +964,17 @@
       </c>
       <c r="M14" s="0" t="inlineStr">
         <is>
-          <t>4500000324202608138809307553</t>
+          <t>4500000383202608135550322726</t>
         </is>
       </c>
     </row>
     <row r="15" spans="1:14">
       <c r="A15" s="0">
-        <v>49196507</v>
+        <v>49197555</v>
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t>香字钟培芷</t>
+          <t>FXH*</t>
         </is>
       </c>
       <c r="C15" s="0" t="inlineStr">
@@ -999,7 +999,7 @@
       </c>
       <c r="G15" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:32:53</t>
+          <t>2026-08-13 21:55:10</t>
         </is>
       </c>
       <c r="H15" s="0" t="inlineStr">
@@ -1029,17 +1029,17 @@
       </c>
       <c r="M15" s="0" t="inlineStr">
         <is>
-          <t>4500000370202608133660294135</t>
+          <t>4500000376202608139667116905</t>
         </is>
       </c>
     </row>
     <row r="16" spans="1:14">
       <c r="A16" s="0">
-        <v>49196498</v>
+        <v>49197551</v>
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t>孟光宗</t>
+          <t>书英</t>
         </is>
       </c>
       <c r="C16" s="0" t="inlineStr">
@@ -1064,7 +1064,7 @@
       </c>
       <c r="G16" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:37:14</t>
+          <t>2026-08-13 21:55:09</t>
         </is>
       </c>
       <c r="H16" s="0" t="inlineStr">
@@ -1094,17 +1094,17 @@
       </c>
       <c r="M16" s="0" t="inlineStr">
         <is>
-          <t>4500000363202608138859211736</t>
+          <t>4500000363202608135183726220</t>
         </is>
       </c>
     </row>
     <row r="17" spans="1:14">
       <c r="A17" s="0">
-        <v>49196495</v>
+        <v>49197500</v>
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t>夏雨晴的妈妈（天发水芹</t>
+          <t>求智慧</t>
         </is>
       </c>
       <c r="C17" s="0" t="inlineStr">
@@ -1129,7 +1129,7 @@
       </c>
       <c r="G17" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:32:41</t>
+          <t>2026-08-13 21:54:20</t>
         </is>
       </c>
       <c r="H17" s="0" t="inlineStr">
@@ -1159,22 +1159,17 @@
       </c>
       <c r="M17" s="0" t="inlineStr">
         <is>
-          <t>4500000371202608138873102820</t>
-        </is>
-      </c>
-      <c r="N17" s="0" t="inlineStr">
-        <is>
-          <t>湾仔区</t>
+          <t>4500000356202608136477567012</t>
         </is>
       </c>
     </row>
     <row r="18" spans="1:14">
       <c r="A18" s="0">
-        <v>49196485</v>
+        <v>49196660</v>
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t>法苑文印广告</t>
+          <t>陈书先</t>
         </is>
       </c>
       <c r="C18" s="0" t="inlineStr">
@@ -1199,7 +1194,7 @@
       </c>
       <c r="G18" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:33:06</t>
+          <t>2026-08-13 21:35:55</t>
         </is>
       </c>
       <c r="H18" s="0" t="inlineStr">
@@ -1229,17 +1224,17 @@
       </c>
       <c r="M18" s="0" t="inlineStr">
         <is>
-          <t>4500000379202608139506557676</t>
+          <t>4500000362202608137513582005</t>
         </is>
       </c>
     </row>
     <row r="19" spans="1:14">
       <c r="A19" s="0">
-        <v>49196481</v>
+        <v>49196649</v>
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t>四季果</t>
+          <t>chenchen</t>
         </is>
       </c>
       <c r="C19" s="0" t="inlineStr">
@@ -1264,7 +1259,7 @@
       </c>
       <c r="G19" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:33:08</t>
+          <t>2026-08-13 21:35:37</t>
         </is>
       </c>
       <c r="H19" s="0" t="inlineStr">
@@ -1294,17 +1289,17 @@
       </c>
       <c r="M19" s="0" t="inlineStr">
         <is>
-          <t>4500000335202608134787426208</t>
+          <t>4500000360202608131193472561</t>
         </is>
       </c>
     </row>
     <row r="20" spans="1:14">
       <c r="A20" s="0">
-        <v>49196479</v>
+        <v>49196616</v>
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t>仇尚妹</t>
+          <t>因子</t>
         </is>
       </c>
       <c r="C20" s="0" t="inlineStr">
@@ -1329,7 +1324,7 @@
       </c>
       <c r="G20" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:32:43</t>
+          <t>2026-08-13 21:35:34</t>
         </is>
       </c>
       <c r="H20" s="0" t="inlineStr">
@@ -1359,17 +1354,17 @@
       </c>
       <c r="M20" s="0" t="inlineStr">
         <is>
-          <t>4500000374202608136810799236</t>
+          <t>4500000381202608131084069069</t>
         </is>
       </c>
     </row>
     <row r="21" spans="1:14">
       <c r="A21" s="0">
-        <v>49196478</v>
+        <v>49196580</v>
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t>A古庄店大新手机卖场库琳琳</t>
+          <t>包容</t>
         </is>
       </c>
       <c r="C21" s="0" t="inlineStr">
@@ -1394,7 +1389,7 @@
       </c>
       <c r="G21" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:32:42</t>
+          <t>2026-08-13 21:34:49</t>
         </is>
       </c>
       <c r="H21" s="0" t="inlineStr">
@@ -1424,17 +1419,17 @@
       </c>
       <c r="M21" s="0" t="inlineStr">
         <is>
-          <t>4500000373202608137311399529</t>
+          <t>4500000329202608134515206220</t>
         </is>
       </c>
     </row>
     <row r="22" spans="1:14">
       <c r="A22" s="0">
-        <v>49196473</v>
+        <v>49196556</v>
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t>刘玉云机械租赁服务部15905691602</t>
+          <t>小芳</t>
         </is>
       </c>
       <c r="C22" s="0" t="inlineStr">
@@ -1459,7 +1454,7 @@
       </c>
       <c r="G22" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:32:30</t>
+          <t>2026-08-13 21:34:00</t>
         </is>
       </c>
       <c r="H22" s="0" t="inlineStr">
@@ -1489,17 +1484,17 @@
       </c>
       <c r="M22" s="0" t="inlineStr">
         <is>
-          <t>4500000315202608134297741797</t>
+          <t>4500000380202608131586040016</t>
         </is>
       </c>
     </row>
     <row r="23" spans="1:14">
       <c r="A23" s="0">
-        <v>49196470</v>
+        <v>49196547</v>
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t>众舍康安二手房丽姐</t>
+          <t>雷宁</t>
         </is>
       </c>
       <c r="C23" s="0" t="inlineStr">
@@ -1524,7 +1519,7 @@
       </c>
       <c r="G23" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:32:28</t>
+          <t>2026-08-13 21:34:30</t>
         </is>
       </c>
       <c r="H23" s="0" t="inlineStr">
@@ -1554,17 +1549,17 @@
       </c>
       <c r="M23" s="0" t="inlineStr">
         <is>
-          <t>4500000325202608137489426707</t>
+          <t>4500000368202608133116145497</t>
         </is>
       </c>
     </row>
     <row r="24" spans="1:14">
       <c r="A24" s="0">
-        <v>49196462</v>
+        <v>49196546</v>
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t>欢欢</t>
+          <t>兰莓</t>
         </is>
       </c>
       <c r="C24" s="0" t="inlineStr">
@@ -1589,7 +1584,7 @@
       </c>
       <c r="G24" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:32:31</t>
+          <t>2026-08-13 21:56:17</t>
         </is>
       </c>
       <c r="H24" s="0" t="inlineStr">
@@ -1619,17 +1614,17 @@
       </c>
       <c r="M24" s="0" t="inlineStr">
         <is>
-          <t>4500000382202608136078541008</t>
+          <t>4500000352202608136989637138</t>
         </is>
       </c>
     </row>
     <row r="25" spans="1:14">
       <c r="A25" s="0">
-        <v>49196456</v>
+        <v>49196528</v>
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>润花</t>
+          <t>赵子睿奶奶</t>
         </is>
       </c>
       <c r="C25" s="0" t="inlineStr">
@@ -1654,7 +1649,7 @@
       </c>
       <c r="G25" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:32:41</t>
+          <t>2026-08-13 21:33:22</t>
         </is>
       </c>
       <c r="H25" s="0" t="inlineStr">
@@ -1684,17 +1679,17 @@
       </c>
       <c r="M25" s="0" t="inlineStr">
         <is>
-          <t>4500000365202608139285322594</t>
+          <t>4500000345202608137236789446</t>
         </is>
       </c>
     </row>
     <row r="26" spans="1:14">
       <c r="A26" s="0">
-        <v>49196455</v>
+        <v>49196510</v>
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t>风之韵</t>
+          <t>山岭巨人</t>
         </is>
       </c>
       <c r="C26" s="0" t="inlineStr">
@@ -1719,7 +1714,7 @@
       </c>
       <c r="G26" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:32:34</t>
+          <t>2026-08-13 21:35:22</t>
         </is>
       </c>
       <c r="H26" s="0" t="inlineStr">
@@ -1749,17 +1744,17 @@
       </c>
       <c r="M26" s="0" t="inlineStr">
         <is>
-          <t>4500000339202608137054529020</t>
+          <t>4500000324202608138809307553</t>
         </is>
       </c>
     </row>
     <row r="27" spans="1:14">
       <c r="A27" s="0">
-        <v>49196452</v>
+        <v>49196507</v>
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>开心每一天</t>
+          <t>香字钟培芷</t>
         </is>
       </c>
       <c r="C27" s="0" t="inlineStr">
@@ -1784,7 +1779,7 @@
       </c>
       <c r="G27" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:32:40</t>
+          <t>2026-08-13 21:32:53</t>
         </is>
       </c>
       <c r="H27" s="0" t="inlineStr">
@@ -1814,22 +1809,17 @@
       </c>
       <c r="M27" s="0" t="inlineStr">
         <is>
-          <t>4500000327202608131603927208</t>
-        </is>
-      </c>
-      <c r="N27" s="0" t="inlineStr">
-        <is>
-          <t>连云港</t>
+          <t>4500000370202608133660294135</t>
         </is>
       </c>
     </row>
     <row r="28" spans="1:14">
       <c r="A28" s="0">
-        <v>49196449</v>
+        <v>49196498</v>
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>吉乐常伴</t>
+          <t>孟光宗</t>
         </is>
       </c>
       <c r="C28" s="0" t="inlineStr">
@@ -1854,7 +1844,7 @@
       </c>
       <c r="G28" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:32:23</t>
+          <t>2026-08-13 21:37:14</t>
         </is>
       </c>
       <c r="H28" s="0" t="inlineStr">
@@ -1884,17 +1874,17 @@
       </c>
       <c r="M28" s="0" t="inlineStr">
         <is>
-          <t>4500000340202608139313739490</t>
+          <t>4500000363202608138859211736</t>
         </is>
       </c>
     </row>
     <row r="29" spans="1:14">
       <c r="A29" s="0">
-        <v>49196445</v>
+        <v>49196495</v>
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t>快乐宝贝</t>
+          <t>夏雨晴的妈妈（天发水芹</t>
         </is>
       </c>
       <c r="C29" s="0" t="inlineStr">
@@ -1919,7 +1909,7 @@
       </c>
       <c r="G29" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:32:15</t>
+          <t>2026-08-13 21:32:41</t>
         </is>
       </c>
       <c r="H29" s="0" t="inlineStr">
@@ -1949,17 +1939,22 @@
       </c>
       <c r="M29" s="0" t="inlineStr">
         <is>
-          <t>4500000326202608133056225424</t>
+          <t>4500000371202608138873102820</t>
+        </is>
+      </c>
+      <c r="N29" s="0" t="inlineStr">
+        <is>
+          <t>湾仔区</t>
         </is>
       </c>
     </row>
     <row r="30" spans="1:14">
       <c r="A30" s="0">
-        <v>49196441</v>
+        <v>49196485</v>
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t>感恩快乐每一天</t>
+          <t>法苑文印广告</t>
         </is>
       </c>
       <c r="C30" s="0" t="inlineStr">
@@ -1984,7 +1979,7 @@
       </c>
       <c r="G30" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:32:13</t>
+          <t>2026-08-13 21:33:06</t>
         </is>
       </c>
       <c r="H30" s="0" t="inlineStr">
@@ -2014,17 +2009,17 @@
       </c>
       <c r="M30" s="0" t="inlineStr">
         <is>
-          <t>4500000383202608132236113522</t>
+          <t>4500000379202608139506557676</t>
         </is>
       </c>
     </row>
     <row r="31" spans="1:14">
       <c r="A31" s="0">
-        <v>49196439</v>
+        <v>49196481</v>
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t>翰林世家京墨18240001035</t>
+          <t>四季果</t>
         </is>
       </c>
       <c r="C31" s="0" t="inlineStr">
@@ -2049,7 +2044,7 @@
       </c>
       <c r="G31" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:32:18</t>
+          <t>2026-08-13 21:33:08</t>
         </is>
       </c>
       <c r="H31" s="0" t="inlineStr">
@@ -2079,17 +2074,17 @@
       </c>
       <c r="M31" s="0" t="inlineStr">
         <is>
-          <t>4500000315202608131410776307</t>
+          <t>4500000335202608134787426208</t>
         </is>
       </c>
     </row>
     <row r="32" spans="1:14">
       <c r="A32" s="0">
-        <v>49196437</v>
+        <v>49196479</v>
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t>悦朵宝贝</t>
+          <t>仇尚妹</t>
         </is>
       </c>
       <c r="C32" s="0" t="inlineStr">
@@ -2114,7 +2109,7 @@
       </c>
       <c r="G32" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:32:06</t>
+          <t>2026-08-13 21:32:43</t>
         </is>
       </c>
       <c r="H32" s="0" t="inlineStr">
@@ -2144,17 +2139,17 @@
       </c>
       <c r="M32" s="0" t="inlineStr">
         <is>
-          <t>4500000343202608135681746747</t>
+          <t>4500000374202608136810799236</t>
         </is>
       </c>
     </row>
     <row r="33" spans="1:14">
       <c r="A33" s="0">
-        <v>49196435</v>
+        <v>49196478</v>
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t>我的幸福</t>
+          <t>A古庄店大新手机卖场库琳琳</t>
         </is>
       </c>
       <c r="C33" s="0" t="inlineStr">
@@ -2179,7 +2174,7 @@
       </c>
       <c r="G33" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:32:23</t>
+          <t>2026-08-13 21:32:42</t>
         </is>
       </c>
       <c r="H33" s="0" t="inlineStr">
@@ -2209,17 +2204,17 @@
       </c>
       <c r="M33" s="0" t="inlineStr">
         <is>
-          <t>4500000331202608138821842807</t>
+          <t>4500000373202608137311399529</t>
         </is>
       </c>
     </row>
     <row r="34" spans="1:14">
       <c r="A34" s="0">
-        <v>49196433</v>
+        <v>49196473</v>
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t>程胜英</t>
+          <t>刘玉云机械租赁服务部15905691602</t>
         </is>
       </c>
       <c r="C34" s="0" t="inlineStr">
@@ -2244,7 +2239,7 @@
       </c>
       <c r="G34" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:32:33</t>
+          <t>2026-08-13 21:32:30</t>
         </is>
       </c>
       <c r="H34" s="0" t="inlineStr">
@@ -2274,17 +2269,17 @@
       </c>
       <c r="M34" s="0" t="inlineStr">
         <is>
-          <t>4500000338202608136558136840</t>
+          <t>4500000315202608134297741797</t>
         </is>
       </c>
     </row>
     <row r="35" spans="1:14">
       <c r="A35" s="0">
-        <v>49196424</v>
+        <v>49196470</v>
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t>甘峰源奶奶</t>
+          <t>众舍康安二手房丽姐</t>
         </is>
       </c>
       <c r="C35" s="0" t="inlineStr">
@@ -2309,7 +2304,7 @@
       </c>
       <c r="G35" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:32:16</t>
+          <t>2026-08-13 21:32:28</t>
         </is>
       </c>
       <c r="H35" s="0" t="inlineStr">
@@ -2339,17 +2334,17 @@
       </c>
       <c r="M35" s="0" t="inlineStr">
         <is>
-          <t>4500000374202608139681236972</t>
+          <t>4500000325202608137489426707</t>
         </is>
       </c>
     </row>
     <row r="36" spans="1:14">
       <c r="A36" s="0">
-        <v>49196412</v>
+        <v>49196462</v>
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>贝贝老妈</t>
+          <t>欢欢</t>
         </is>
       </c>
       <c r="C36" s="0" t="inlineStr">
@@ -2374,7 +2369,7 @@
       </c>
       <c r="G36" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:31:49</t>
+          <t>2026-08-13 21:32:31</t>
         </is>
       </c>
       <c r="H36" s="0" t="inlineStr">
@@ -2404,17 +2399,17 @@
       </c>
       <c r="M36" s="0" t="inlineStr">
         <is>
-          <t>4500000360202608138627203805</t>
+          <t>4500000382202608136078541008</t>
         </is>
       </c>
     </row>
     <row r="37" spans="1:14">
       <c r="A37" s="0">
-        <v>49196406</v>
+        <v>49196456</v>
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t>过好每一天</t>
+          <t>润花</t>
         </is>
       </c>
       <c r="C37" s="0" t="inlineStr">
@@ -2439,7 +2434,7 @@
       </c>
       <c r="G37" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:31:55</t>
+          <t>2026-08-13 21:32:41</t>
         </is>
       </c>
       <c r="H37" s="0" t="inlineStr">
@@ -2469,17 +2464,17 @@
       </c>
       <c r="M37" s="0" t="inlineStr">
         <is>
-          <t>4500000384202608139484061741</t>
+          <t>4500000365202608139285322594</t>
         </is>
       </c>
     </row>
     <row r="38" spans="1:14">
       <c r="A38" s="0">
-        <v>49196403</v>
+        <v>49196455</v>
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>迪迪</t>
+          <t>风之韵</t>
         </is>
       </c>
       <c r="C38" s="0" t="inlineStr">
@@ -2504,7 +2499,7 @@
       </c>
       <c r="G38" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:31:58</t>
+          <t>2026-08-13 21:32:34</t>
         </is>
       </c>
       <c r="H38" s="0" t="inlineStr">
@@ -2534,17 +2529,17 @@
       </c>
       <c r="M38" s="0" t="inlineStr">
         <is>
-          <t>4500000326202608138209731181</t>
+          <t>4500000339202608137054529020</t>
         </is>
       </c>
     </row>
     <row r="39" spans="1:14">
       <c r="A39" s="0">
-        <v>49196399</v>
+        <v>49196452</v>
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>境随心转</t>
+          <t>开心每一天</t>
         </is>
       </c>
       <c r="C39" s="0" t="inlineStr">
@@ -2569,7 +2564,7 @@
       </c>
       <c r="G39" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:31:47</t>
+          <t>2026-08-13 21:32:40</t>
         </is>
       </c>
       <c r="H39" s="0" t="inlineStr">
@@ -2599,17 +2594,22 @@
       </c>
       <c r="M39" s="0" t="inlineStr">
         <is>
-          <t>4500000380202608138946210876</t>
+          <t>4500000327202608131603927208</t>
+        </is>
+      </c>
+      <c r="N39" s="0" t="inlineStr">
+        <is>
+          <t>连云港</t>
         </is>
       </c>
     </row>
     <row r="40" spans="1:14">
       <c r="A40" s="0">
-        <v>49196391</v>
+        <v>49196449</v>
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>💖海霞💖</t>
+          <t>吉乐常伴</t>
         </is>
       </c>
       <c r="C40" s="0" t="inlineStr">
@@ -2634,7 +2634,7 @@
       </c>
       <c r="G40" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:32:01</t>
+          <t>2026-08-13 21:32:23</t>
         </is>
       </c>
       <c r="H40" s="0" t="inlineStr">
@@ -2664,17 +2664,17 @@
       </c>
       <c r="M40" s="0" t="inlineStr">
         <is>
-          <t>4500000326202608133672869122</t>
+          <t>4500000340202608139313739490</t>
         </is>
       </c>
     </row>
     <row r="41" spans="1:14">
       <c r="A41" s="0">
-        <v>49196390</v>
+        <v>49196445</v>
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t>翠翠</t>
+          <t>快乐宝贝</t>
         </is>
       </c>
       <c r="C41" s="0" t="inlineStr">
@@ -2699,7 +2699,7 @@
       </c>
       <c r="G41" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:31:38</t>
+          <t>2026-08-13 21:32:15</t>
         </is>
       </c>
       <c r="H41" s="0" t="inlineStr">
@@ -2729,22 +2729,17 @@
       </c>
       <c r="M41" s="0" t="inlineStr">
         <is>
-          <t>4500000351202608139683947334</t>
-        </is>
-      </c>
-      <c r="N41" s="0" t="inlineStr">
-        <is>
-          <t>广州</t>
+          <t>4500000326202608133056225424</t>
         </is>
       </c>
     </row>
     <row r="42" spans="1:14">
       <c r="A42" s="0">
-        <v>49196389</v>
+        <v>49196441</v>
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t>漫步繁华街</t>
+          <t>感恩快乐每一天</t>
         </is>
       </c>
       <c r="C42" s="0" t="inlineStr">
@@ -2769,7 +2764,7 @@
       </c>
       <c r="G42" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:32:39</t>
+          <t>2026-08-13 21:32:13</t>
         </is>
       </c>
       <c r="H42" s="0" t="inlineStr">
@@ -2799,17 +2794,17 @@
       </c>
       <c r="M42" s="0" t="inlineStr">
         <is>
-          <t>4500000375202608135974835236</t>
+          <t>4500000383202608132236113522</t>
         </is>
       </c>
     </row>
     <row r="43" spans="1:14">
       <c r="A43" s="0">
-        <v>49196385</v>
+        <v>49196439</v>
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t>平淡人生🌲</t>
+          <t>翰林世家京墨18240001035</t>
         </is>
       </c>
       <c r="C43" s="0" t="inlineStr">
@@ -2834,7 +2829,7 @@
       </c>
       <c r="G43" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:31:35</t>
+          <t>2026-08-13 21:32:18</t>
         </is>
       </c>
       <c r="H43" s="0" t="inlineStr">
@@ -2864,17 +2859,17 @@
       </c>
       <c r="M43" s="0" t="inlineStr">
         <is>
-          <t>4500000359202608136587117638</t>
+          <t>4500000315202608131410776307</t>
         </is>
       </c>
     </row>
     <row r="44" spans="1:14">
       <c r="A44" s="0">
-        <v>49196384</v>
+        <v>49196437</v>
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t>眼镜灯饰城3楼76号15923959748</t>
+          <t>悦朵宝贝</t>
         </is>
       </c>
       <c r="C44" s="0" t="inlineStr">
@@ -2899,7 +2894,7 @@
       </c>
       <c r="G44" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:31:34</t>
+          <t>2026-08-13 21:32:06</t>
         </is>
       </c>
       <c r="H44" s="0" t="inlineStr">
@@ -2929,17 +2924,17 @@
       </c>
       <c r="M44" s="0" t="inlineStr">
         <is>
-          <t>4500000333202608139966140440</t>
+          <t>4500000343202608135681746747</t>
         </is>
       </c>
     </row>
     <row r="45" spans="1:14">
       <c r="A45" s="0">
-        <v>49196383</v>
+        <v>49196435</v>
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t>喜枝</t>
+          <t>我的幸福</t>
         </is>
       </c>
       <c r="C45" s="0" t="inlineStr">
@@ -2964,7 +2959,7 @@
       </c>
       <c r="G45" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13 21:31:45</t>
+          <t>2026-08-13 21:32:23</t>
         </is>
       </c>
       <c r="H45" s="0" t="inlineStr">
@@ -2994,17 +2989,17 @@
       </c>
       <c r="M45" s="0" t="inlineStr">
         <is>
-          <t>4500000333202608138694510811</t>
+          <t>4500000331202608138821842807</t>
         </is>
       </c>
     </row>
     <row r="46" spans="1:14">
       <c r="A46" s="0">
-        <v>49155446</v>
+        <v>49196433</v>
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t>笑口常开</t>
+          <t>程胜英</t>
         </is>
       </c>
       <c r="C46" s="0" t="inlineStr">
@@ -3029,7 +3024,7 @@
       </c>
       <c r="G46" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:36:06</t>
+          <t>2026-08-13 21:32:33</t>
         </is>
       </c>
       <c r="H46" s="0" t="inlineStr">
@@ -3059,17 +3054,17 @@
       </c>
       <c r="M46" s="0" t="inlineStr">
         <is>
-          <t>4500000376202608121856487760</t>
+          <t>4500000338202608136558136840</t>
         </is>
       </c>
     </row>
     <row r="47" spans="1:14">
       <c r="A47" s="0">
-        <v>49155389</v>
+        <v>49196424</v>
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t>奥普郭彦丽13937990394</t>
+          <t>甘峰源奶奶</t>
         </is>
       </c>
       <c r="C47" s="0" t="inlineStr">
@@ -3094,7 +3089,7 @@
       </c>
       <c r="G47" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:35:44</t>
+          <t>2026-08-13 21:32:16</t>
         </is>
       </c>
       <c r="H47" s="0" t="inlineStr">
@@ -3124,17 +3119,17 @@
       </c>
       <c r="M47" s="0" t="inlineStr">
         <is>
-          <t>4500000324202608124582542642</t>
+          <t>4500000374202608139681236972</t>
         </is>
       </c>
     </row>
     <row r="48" spans="1:14">
       <c r="A48" s="0">
-        <v>49155374</v>
+        <v>49196412</v>
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t>流星雨文华</t>
+          <t>贝贝老妈</t>
         </is>
       </c>
       <c r="C48" s="0" t="inlineStr">
@@ -3159,7 +3154,7 @@
       </c>
       <c r="G48" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:35:26</t>
+          <t>2026-08-13 21:31:49</t>
         </is>
       </c>
       <c r="H48" s="0" t="inlineStr">
@@ -3189,17 +3184,17 @@
       </c>
       <c r="M48" s="0" t="inlineStr">
         <is>
-          <t>4500000377202608121430434820</t>
+          <t>4500000360202608138627203805</t>
         </is>
       </c>
     </row>
     <row r="49" spans="1:14">
       <c r="A49" s="0">
-        <v>49155368</v>
+        <v>49196406</v>
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t>笑对人生</t>
+          <t>过好每一天</t>
         </is>
       </c>
       <c r="C49" s="0" t="inlineStr">
@@ -3224,7 +3219,7 @@
       </c>
       <c r="G49" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:34:56</t>
+          <t>2026-08-13 21:31:55</t>
         </is>
       </c>
       <c r="H49" s="0" t="inlineStr">
@@ -3254,17 +3249,17 @@
       </c>
       <c r="M49" s="0" t="inlineStr">
         <is>
-          <t>4500000316202608126193240482</t>
+          <t>4500000384202608139484061741</t>
         </is>
       </c>
     </row>
     <row r="50" spans="1:14">
       <c r="A50" s="0">
-        <v>49155365</v>
+        <v>49196403</v>
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t>秀</t>
+          <t>迪迪</t>
         </is>
       </c>
       <c r="C50" s="0" t="inlineStr">
@@ -3289,7 +3284,7 @@
       </c>
       <c r="G50" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:34:41</t>
+          <t>2026-08-13 21:31:58</t>
         </is>
       </c>
       <c r="H50" s="0" t="inlineStr">
@@ -3319,17 +3314,17 @@
       </c>
       <c r="M50" s="0" t="inlineStr">
         <is>
-          <t>4500000363202608121090433848</t>
+          <t>4500000326202608138209731181</t>
         </is>
       </c>
     </row>
     <row r="51" spans="1:14">
       <c r="A51" s="0">
-        <v>49155364</v>
+        <v>49196399</v>
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t>冯衣制版18966913385</t>
+          <t>境随心转</t>
         </is>
       </c>
       <c r="C51" s="0" t="inlineStr">
@@ -3354,7 +3349,7 @@
       </c>
       <c r="G51" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:35:09</t>
+          <t>2026-08-13 21:31:47</t>
         </is>
       </c>
       <c r="H51" s="0" t="inlineStr">
@@ -3384,17 +3379,17 @@
       </c>
       <c r="M51" s="0" t="inlineStr">
         <is>
-          <t>4500000348202608122728123344</t>
+          <t>4500000380202608138946210876</t>
         </is>
       </c>
     </row>
     <row r="52" spans="1:14">
       <c r="A52" s="0">
-        <v>49155363</v>
+        <v>49196391</v>
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t>平安</t>
+          <t>💖海霞💖</t>
         </is>
       </c>
       <c r="C52" s="0" t="inlineStr">
@@ -3419,7 +3414,7 @@
       </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:34:54</t>
+          <t>2026-08-13 21:32:01</t>
         </is>
       </c>
       <c r="H52" s="0" t="inlineStr">
@@ -3449,17 +3444,17 @@
       </c>
       <c r="M52" s="0" t="inlineStr">
         <is>
-          <t>4500000320202608128317430099</t>
+          <t>4500000326202608133672869122</t>
         </is>
       </c>
     </row>
     <row r="53" spans="1:14">
       <c r="A53" s="0">
-        <v>49155361</v>
+        <v>49196390</v>
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t>春华秋实</t>
+          <t>翠翠</t>
         </is>
       </c>
       <c r="C53" s="0" t="inlineStr">
@@ -3484,7 +3479,7 @@
       </c>
       <c r="G53" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:34:48</t>
+          <t>2026-08-13 21:31:38</t>
         </is>
       </c>
       <c r="H53" s="0" t="inlineStr">
@@ -3514,17 +3509,22 @@
       </c>
       <c r="M53" s="0" t="inlineStr">
         <is>
-          <t>4500000346202608121174096033</t>
+          <t>4500000351202608139683947334</t>
+        </is>
+      </c>
+      <c r="N53" s="0" t="inlineStr">
+        <is>
+          <t>广州</t>
         </is>
       </c>
     </row>
     <row r="54" spans="1:14">
       <c r="A54" s="0">
-        <v>49155359</v>
+        <v>49196389</v>
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t>春梅。</t>
+          <t>漫步繁华街</t>
         </is>
       </c>
       <c r="C54" s="0" t="inlineStr">
@@ -3549,7 +3549,7 @@
       </c>
       <c r="G54" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:34:36</t>
+          <t>2026-08-13 21:32:39</t>
         </is>
       </c>
       <c r="H54" s="0" t="inlineStr">
@@ -3579,17 +3579,17 @@
       </c>
       <c r="M54" s="0" t="inlineStr">
         <is>
-          <t>4500000374202608123637081551</t>
+          <t>4500000375202608135974835236</t>
         </is>
       </c>
     </row>
     <row r="55" spans="1:14">
       <c r="A55" s="0">
-        <v>49155344</v>
+        <v>49196385</v>
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t>自由人生</t>
+          <t>平淡人生🌲</t>
         </is>
       </c>
       <c r="C55" s="0" t="inlineStr">
@@ -3614,7 +3614,7 @@
       </c>
       <c r="G55" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:34:25</t>
+          <t>2026-08-13 21:31:35</t>
         </is>
       </c>
       <c r="H55" s="0" t="inlineStr">
@@ -3644,17 +3644,17 @@
       </c>
       <c r="M55" s="0" t="inlineStr">
         <is>
-          <t>4500000317202608129865186226</t>
+          <t>4500000359202608136587117638</t>
         </is>
       </c>
     </row>
     <row r="56" spans="1:14">
       <c r="A56" s="0">
-        <v>49155337</v>
+        <v>49196384</v>
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t>红红</t>
+          <t>眼镜灯饰城3楼76号15923959748</t>
         </is>
       </c>
       <c r="C56" s="0" t="inlineStr">
@@ -3679,7 +3679,7 @@
       </c>
       <c r="G56" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:34:50</t>
+          <t>2026-08-13 21:31:34</t>
         </is>
       </c>
       <c r="H56" s="0" t="inlineStr">
@@ -3709,17 +3709,17 @@
       </c>
       <c r="M56" s="0" t="inlineStr">
         <is>
-          <t>4500000327202608125530964720</t>
+          <t>4500000333202608139966140440</t>
         </is>
       </c>
     </row>
     <row r="57" spans="1:14">
       <c r="A57" s="0">
-        <v>49155330</v>
+        <v>49196383</v>
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t>徐淑香</t>
+          <t>喜枝</t>
         </is>
       </c>
       <c r="C57" s="0" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:34:20</t>
+          <t>2026-08-13 21:31:45</t>
         </is>
       </c>
       <c r="H57" s="0" t="inlineStr">
@@ -3774,17 +3774,17 @@
       </c>
       <c r="M57" s="0" t="inlineStr">
         <is>
-          <t>4500000359202608124983971576</t>
+          <t>4500000333202608138694510811</t>
         </is>
       </c>
     </row>
     <row r="58" spans="1:14">
       <c r="A58" s="0">
-        <v>49155314</v>
+        <v>49155446</v>
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t>H叶</t>
+          <t>笑口常开</t>
         </is>
       </c>
       <c r="C58" s="0" t="inlineStr">
@@ -3809,7 +3809,7 @@
       </c>
       <c r="G58" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:33:57</t>
+          <t>2026-08-12 21:36:06</t>
         </is>
       </c>
       <c r="H58" s="0" t="inlineStr">
@@ -3839,17 +3839,17 @@
       </c>
       <c r="M58" s="0" t="inlineStr">
         <is>
-          <t>4500000322202608128162955185</t>
+          <t>4500000376202608121856487760</t>
         </is>
       </c>
     </row>
     <row r="59" spans="1:14">
       <c r="A59" s="0">
-        <v>49155309</v>
+        <v>49155389</v>
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t>A0000刘氏修脚红姐</t>
+          <t>奥普郭彦丽13937990394</t>
         </is>
       </c>
       <c r="C59" s="0" t="inlineStr">
@@ -3874,7 +3874,7 @@
       </c>
       <c r="G59" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:33:47</t>
+          <t>2026-08-12 21:35:44</t>
         </is>
       </c>
       <c r="H59" s="0" t="inlineStr">
@@ -3904,17 +3904,17 @@
       </c>
       <c r="M59" s="0" t="inlineStr">
         <is>
-          <t>4500000333202608127176361921</t>
+          <t>4500000324202608124582542642</t>
         </is>
       </c>
     </row>
     <row r="60" spans="1:14">
       <c r="A60" s="0">
-        <v>49155304</v>
+        <v>49155374</v>
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t>万树红</t>
+          <t>流星雨文华</t>
         </is>
       </c>
       <c r="C60" s="0" t="inlineStr">
@@ -3939,7 +3939,7 @@
       </c>
       <c r="G60" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:33:52</t>
+          <t>2026-08-12 21:35:26</t>
         </is>
       </c>
       <c r="H60" s="0" t="inlineStr">
@@ -3969,17 +3969,17 @@
       </c>
       <c r="M60" s="0" t="inlineStr">
         <is>
-          <t>4500000379202608123430987084</t>
+          <t>4500000377202608121430434820</t>
         </is>
       </c>
     </row>
     <row r="61" spans="1:14">
       <c r="A61" s="0">
-        <v>49155293</v>
+        <v>49155368</v>
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t>往事如烟</t>
+          <t>笑对人生</t>
         </is>
       </c>
       <c r="C61" s="0" t="inlineStr">
@@ -4004,7 +4004,7 @@
       </c>
       <c r="G61" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:33:33</t>
+          <t>2026-08-12 21:34:56</t>
         </is>
       </c>
       <c r="H61" s="0" t="inlineStr">
@@ -4034,17 +4034,17 @@
       </c>
       <c r="M61" s="0" t="inlineStr">
         <is>
-          <t>4500000360202608121388094535</t>
+          <t>4500000316202608126193240482</t>
         </is>
       </c>
     </row>
     <row r="62" spans="1:14">
       <c r="A62" s="0">
-        <v>49155283</v>
+        <v>49155365</v>
       </c>
       <c r="B62" s="0" t="inlineStr">
         <is>
-          <t>雪洁</t>
+          <t>秀</t>
         </is>
       </c>
       <c r="C62" s="0" t="inlineStr">
@@ -4069,7 +4069,7 @@
       </c>
       <c r="G62" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:33:27</t>
+          <t>2026-08-12 21:34:41</t>
         </is>
       </c>
       <c r="H62" s="0" t="inlineStr">
@@ -4099,17 +4099,17 @@
       </c>
       <c r="M62" s="0" t="inlineStr">
         <is>
-          <t>4500000369202608125072492429</t>
+          <t>4500000363202608121090433848</t>
         </is>
       </c>
     </row>
     <row r="63" spans="1:14">
       <c r="A63" s="0">
-        <v>49155274</v>
+        <v>49155364</v>
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
-          <t>文英</t>
+          <t>冯衣制版18966913385</t>
         </is>
       </c>
       <c r="C63" s="0" t="inlineStr">
@@ -4134,7 +4134,7 @@
       </c>
       <c r="G63" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:33:24</t>
+          <t>2026-08-12 21:35:09</t>
         </is>
       </c>
       <c r="H63" s="0" t="inlineStr">
@@ -4164,17 +4164,17 @@
       </c>
       <c r="M63" s="0" t="inlineStr">
         <is>
-          <t>4500000373202608127495955817</t>
+          <t>4500000348202608122728123344</t>
         </is>
       </c>
     </row>
     <row r="64" spans="1:14">
       <c r="A64" s="0">
-        <v>49155273</v>
+        <v>49155363</v>
       </c>
       <c r="B64" s="0" t="inlineStr">
         <is>
-          <t>宫本江</t>
+          <t>平安</t>
         </is>
       </c>
       <c r="C64" s="0" t="inlineStr">
@@ -4199,7 +4199,7 @@
       </c>
       <c r="G64" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:33:16</t>
+          <t>2026-08-12 21:34:54</t>
         </is>
       </c>
       <c r="H64" s="0" t="inlineStr">
@@ -4229,17 +4229,17 @@
       </c>
       <c r="M64" s="0" t="inlineStr">
         <is>
-          <t>4500000346202608122111396208</t>
+          <t>4500000320202608128317430099</t>
         </is>
       </c>
     </row>
     <row r="65" spans="1:14">
       <c r="A65" s="0">
-        <v>49155272</v>
+        <v>49155361</v>
       </c>
       <c r="B65" s="0" t="inlineStr">
         <is>
-          <t>悠闲的人</t>
+          <t>春华秋实</t>
         </is>
       </c>
       <c r="C65" s="0" t="inlineStr">
@@ -4264,7 +4264,7 @@
       </c>
       <c r="G65" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:33:13</t>
+          <t>2026-08-12 21:34:48</t>
         </is>
       </c>
       <c r="H65" s="0" t="inlineStr">
@@ -4294,17 +4294,17 @@
       </c>
       <c r="M65" s="0" t="inlineStr">
         <is>
-          <t>4500000331202608122303219210</t>
+          <t>4500000346202608121174096033</t>
         </is>
       </c>
     </row>
     <row r="66" spans="1:14">
       <c r="A66" s="0">
-        <v>49155271</v>
+        <v>49155359</v>
       </c>
       <c r="B66" s="0" t="inlineStr">
         <is>
-          <t>幸福人生</t>
+          <t>春梅。</t>
         </is>
       </c>
       <c r="C66" s="0" t="inlineStr">
@@ -4329,7 +4329,7 @@
       </c>
       <c r="G66" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:34:08</t>
+          <t>2026-08-12 21:34:36</t>
         </is>
       </c>
       <c r="H66" s="0" t="inlineStr">
@@ -4359,17 +4359,17 @@
       </c>
       <c r="M66" s="0" t="inlineStr">
         <is>
-          <t>4500000333202608124799146350</t>
+          <t>4500000374202608123637081551</t>
         </is>
       </c>
     </row>
     <row r="67" spans="1:14">
       <c r="A67" s="0">
-        <v>49155270</v>
+        <v>49155344</v>
       </c>
       <c r="B67" s="0" t="inlineStr">
         <is>
-          <t>雾里看花</t>
+          <t>自由人生</t>
         </is>
       </c>
       <c r="C67" s="0" t="inlineStr">
@@ -4394,7 +4394,7 @@
       </c>
       <c r="G67" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:33:15</t>
+          <t>2026-08-12 21:34:25</t>
         </is>
       </c>
       <c r="H67" s="0" t="inlineStr">
@@ -4424,17 +4424,17 @@
       </c>
       <c r="M67" s="0" t="inlineStr">
         <is>
-          <t>4500000331202608123995555310</t>
+          <t>4500000317202608129865186226</t>
         </is>
       </c>
     </row>
     <row r="68" spans="1:14">
       <c r="A68" s="0">
-        <v>49155266</v>
+        <v>49155337</v>
       </c>
       <c r="B68" s="0" t="inlineStr">
         <is>
-          <t>清风绕指柔</t>
+          <t>红红</t>
         </is>
       </c>
       <c r="C68" s="0" t="inlineStr">
@@ -4459,7 +4459,7 @@
       </c>
       <c r="G68" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:33:31</t>
+          <t>2026-08-12 21:34:50</t>
         </is>
       </c>
       <c r="H68" s="0" t="inlineStr">
@@ -4489,17 +4489,17 @@
       </c>
       <c r="M68" s="0" t="inlineStr">
         <is>
-          <t>4500000333202608127946689166</t>
+          <t>4500000327202608125530964720</t>
         </is>
       </c>
     </row>
     <row r="69" spans="1:14">
       <c r="A69" s="0">
-        <v>49155265</v>
+        <v>49155330</v>
       </c>
       <c r="B69" s="0" t="inlineStr">
         <is>
-          <t>心想事成南无阿弥陀佛</t>
+          <t>徐淑香</t>
         </is>
       </c>
       <c r="C69" s="0" t="inlineStr">
@@ -4524,7 +4524,7 @@
       </c>
       <c r="G69" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:33:42</t>
+          <t>2026-08-12 21:34:20</t>
         </is>
       </c>
       <c r="H69" s="0" t="inlineStr">
@@ -4554,17 +4554,17 @@
       </c>
       <c r="M69" s="0" t="inlineStr">
         <is>
-          <t>4500000330202608126996164764</t>
+          <t>4500000359202608124983971576</t>
         </is>
       </c>
     </row>
     <row r="70" spans="1:14">
       <c r="A70" s="0">
-        <v>49155264</v>
+        <v>49155314</v>
       </c>
       <c r="B70" s="0" t="inlineStr">
         <is>
-          <t>刘凤辉</t>
+          <t>H叶</t>
         </is>
       </c>
       <c r="C70" s="0" t="inlineStr">
@@ -4589,7 +4589,7 @@
       </c>
       <c r="G70" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:33:16</t>
+          <t>2026-08-12 21:33:57</t>
         </is>
       </c>
       <c r="H70" s="0" t="inlineStr">
@@ -4619,17 +4619,17 @@
       </c>
       <c r="M70" s="0" t="inlineStr">
         <is>
-          <t>4500000330202608124680304775</t>
+          <t>4500000322202608128162955185</t>
         </is>
       </c>
     </row>
     <row r="71" spans="1:14">
       <c r="A71" s="0">
-        <v>49155263</v>
+        <v>49155309</v>
       </c>
       <c r="B71" s="0" t="inlineStr">
         <is>
-          <t>朱叶</t>
+          <t>A0000刘氏修脚红姐</t>
         </is>
       </c>
       <c r="C71" s="0" t="inlineStr">
@@ -4654,7 +4654,7 @@
       </c>
       <c r="G71" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:33:18</t>
+          <t>2026-08-12 21:33:47</t>
         </is>
       </c>
       <c r="H71" s="0" t="inlineStr">
@@ -4684,17 +4684,17 @@
       </c>
       <c r="M71" s="0" t="inlineStr">
         <is>
-          <t>4500000345202608124445297817</t>
+          <t>4500000333202608127176361921</t>
         </is>
       </c>
     </row>
     <row r="72" spans="1:14">
       <c r="A72" s="0">
-        <v>49155253</v>
+        <v>49155304</v>
       </c>
       <c r="B72" s="0" t="inlineStr">
         <is>
-          <t>一顺百顺。好运来</t>
+          <t>万树红</t>
         </is>
       </c>
       <c r="C72" s="0" t="inlineStr">
@@ -4719,7 +4719,7 @@
       </c>
       <c r="G72" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:33:51</t>
+          <t>2026-08-12 21:33:52</t>
         </is>
       </c>
       <c r="H72" s="0" t="inlineStr">
@@ -4749,17 +4749,17 @@
       </c>
       <c r="M72" s="0" t="inlineStr">
         <is>
-          <t>4500000326202608122909608257</t>
+          <t>4500000379202608123430987084</t>
         </is>
       </c>
     </row>
     <row r="73" spans="1:14">
       <c r="A73" s="0">
-        <v>49155246</v>
+        <v>49155293</v>
       </c>
       <c r="B73" s="0" t="inlineStr">
         <is>
-          <t>陈桂芳</t>
+          <t>往事如烟</t>
         </is>
       </c>
       <c r="C73" s="0" t="inlineStr">
@@ -4784,7 +4784,7 @@
       </c>
       <c r="G73" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:33:14</t>
+          <t>2026-08-12 21:33:33</t>
         </is>
       </c>
       <c r="H73" s="0" t="inlineStr">
@@ -4814,17 +4814,17 @@
       </c>
       <c r="M73" s="0" t="inlineStr">
         <is>
-          <t>4500000378202608126828589764</t>
+          <t>4500000360202608121388094535</t>
         </is>
       </c>
     </row>
     <row r="74" spans="1:14">
       <c r="A74" s="0">
-        <v>49155234</v>
+        <v>49155283</v>
       </c>
       <c r="B74" s="0" t="inlineStr">
         <is>
-          <t>黄仲芬15683592716</t>
+          <t>雪洁</t>
         </is>
       </c>
       <c r="C74" s="0" t="inlineStr">
@@ -4849,7 +4849,7 @@
       </c>
       <c r="G74" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:33:02</t>
+          <t>2026-08-12 21:33:27</t>
         </is>
       </c>
       <c r="H74" s="0" t="inlineStr">
@@ -4879,17 +4879,17 @@
       </c>
       <c r="M74" s="0" t="inlineStr">
         <is>
-          <t>4500000325202608129237945248</t>
+          <t>4500000369202608125072492429</t>
         </is>
       </c>
     </row>
     <row r="75" spans="1:14">
       <c r="A75" s="0">
-        <v>49155233</v>
+        <v>49155274</v>
       </c>
       <c r="B75" s="0" t="inlineStr">
         <is>
-          <t>幸福姐赵会玲</t>
+          <t>文英</t>
         </is>
       </c>
       <c r="C75" s="0" t="inlineStr">
@@ -4914,7 +4914,7 @@
       </c>
       <c r="G75" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:34:04</t>
+          <t>2026-08-12 21:33:24</t>
         </is>
       </c>
       <c r="H75" s="0" t="inlineStr">
@@ -4944,17 +4944,17 @@
       </c>
       <c r="M75" s="0" t="inlineStr">
         <is>
-          <t>4500000317202608128379976752</t>
+          <t>4500000373202608127495955817</t>
         </is>
       </c>
     </row>
     <row r="76" spans="1:14">
       <c r="A76" s="0">
-        <v>49155230</v>
+        <v>49155273</v>
       </c>
       <c r="B76" s="0" t="inlineStr">
         <is>
-          <t>锦鲤果果</t>
+          <t>宫本江</t>
         </is>
       </c>
       <c r="C76" s="0" t="inlineStr">
@@ -4979,7 +4979,7 @@
       </c>
       <c r="G76" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:33:20</t>
+          <t>2026-08-12 21:33:16</t>
         </is>
       </c>
       <c r="H76" s="0" t="inlineStr">
@@ -5009,17 +5009,17 @@
       </c>
       <c r="M76" s="0" t="inlineStr">
         <is>
-          <t>4500000322202608129199323858</t>
+          <t>4500000346202608122111396208</t>
         </is>
       </c>
     </row>
     <row r="77" spans="1:14">
       <c r="A77" s="0">
-        <v>49155226</v>
+        <v>49155272</v>
       </c>
       <c r="B77" s="0" t="inlineStr">
         <is>
-          <t>戎戎</t>
+          <t>悠闲的人</t>
         </is>
       </c>
       <c r="C77" s="0" t="inlineStr">
@@ -5044,7 +5044,7 @@
       </c>
       <c r="G77" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:33:05</t>
+          <t>2026-08-12 21:33:13</t>
         </is>
       </c>
       <c r="H77" s="0" t="inlineStr">
@@ -5074,17 +5074,17 @@
       </c>
       <c r="M77" s="0" t="inlineStr">
         <is>
-          <t>4500000331202608125827170254</t>
+          <t>4500000331202608122303219210</t>
         </is>
       </c>
     </row>
     <row r="78" spans="1:14">
       <c r="A78" s="0">
-        <v>49155220</v>
+        <v>49155271</v>
       </c>
       <c r="B78" s="0" t="inlineStr">
         <is>
-          <t>阿玉</t>
+          <t>幸福人生</t>
         </is>
       </c>
       <c r="C78" s="0" t="inlineStr">
@@ -5109,7 +5109,7 @@
       </c>
       <c r="G78" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:33:16</t>
+          <t>2026-08-12 21:34:08</t>
         </is>
       </c>
       <c r="H78" s="0" t="inlineStr">
@@ -5139,17 +5139,17 @@
       </c>
       <c r="M78" s="0" t="inlineStr">
         <is>
-          <t>4500000345202608129272259118</t>
+          <t>4500000333202608124799146350</t>
         </is>
       </c>
     </row>
     <row r="79" spans="1:14">
       <c r="A79" s="0">
-        <v>49155219</v>
+        <v>49155270</v>
       </c>
       <c r="B79" s="0" t="inlineStr">
         <is>
-          <t>沉淀、</t>
+          <t>雾里看花</t>
         </is>
       </c>
       <c r="C79" s="0" t="inlineStr">
@@ -5174,7 +5174,7 @@
       </c>
       <c r="G79" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:32:56</t>
+          <t>2026-08-12 21:33:15</t>
         </is>
       </c>
       <c r="H79" s="0" t="inlineStr">
@@ -5204,17 +5204,17 @@
       </c>
       <c r="M79" s="0" t="inlineStr">
         <is>
-          <t>4500000372202608124305947387</t>
+          <t>4500000331202608123995555310</t>
         </is>
       </c>
     </row>
     <row r="80" spans="1:14">
       <c r="A80" s="0">
-        <v>49155216</v>
+        <v>49155266</v>
       </c>
       <c r="B80" s="0" t="inlineStr">
         <is>
-          <t>晴天</t>
+          <t>清风绕指柔</t>
         </is>
       </c>
       <c r="C80" s="0" t="inlineStr">
@@ -5239,7 +5239,7 @@
       </c>
       <c r="G80" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:33:07</t>
+          <t>2026-08-12 21:33:31</t>
         </is>
       </c>
       <c r="H80" s="0" t="inlineStr">
@@ -5269,17 +5269,17 @@
       </c>
       <c r="M80" s="0" t="inlineStr">
         <is>
-          <t>4500000334202608122833385690</t>
+          <t>4500000333202608127946689166</t>
         </is>
       </c>
     </row>
     <row r="81" spans="1:14">
       <c r="A81" s="0">
-        <v>49155210</v>
+        <v>49155265</v>
       </c>
       <c r="B81" s="0" t="inlineStr">
         <is>
-          <t>开正商行</t>
+          <t>心想事成南无阿弥陀佛</t>
         </is>
       </c>
       <c r="C81" s="0" t="inlineStr">
@@ -5304,7 +5304,7 @@
       </c>
       <c r="G81" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:33:02</t>
+          <t>2026-08-12 21:33:42</t>
         </is>
       </c>
       <c r="H81" s="0" t="inlineStr">
@@ -5334,17 +5334,17 @@
       </c>
       <c r="M81" s="0" t="inlineStr">
         <is>
-          <t>4500000348202608127466098812</t>
+          <t>4500000330202608126996164764</t>
         </is>
       </c>
     </row>
     <row r="82" spans="1:14">
       <c r="A82" s="0">
-        <v>49155208</v>
+        <v>49155264</v>
       </c>
       <c r="B82" s="0" t="inlineStr">
         <is>
-          <t>傻傻的幸福</t>
+          <t>刘凤辉</t>
         </is>
       </c>
       <c r="C82" s="0" t="inlineStr">
@@ -5369,7 +5369,7 @@
       </c>
       <c r="G82" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:32:54</t>
+          <t>2026-08-12 21:33:16</t>
         </is>
       </c>
       <c r="H82" s="0" t="inlineStr">
@@ -5399,17 +5399,17 @@
       </c>
       <c r="M82" s="0" t="inlineStr">
         <is>
-          <t>4500000378202608122593720010</t>
+          <t>4500000330202608124680304775</t>
         </is>
       </c>
     </row>
     <row r="83" spans="1:14">
       <c r="A83" s="0">
-        <v>49155205</v>
+        <v>49155263</v>
       </c>
       <c r="B83" s="0" t="inlineStr">
         <is>
-          <t>你好</t>
+          <t>朱叶</t>
         </is>
       </c>
       <c r="C83" s="0" t="inlineStr">
@@ -5434,7 +5434,7 @@
       </c>
       <c r="G83" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:32:59</t>
+          <t>2026-08-12 21:33:18</t>
         </is>
       </c>
       <c r="H83" s="0" t="inlineStr">
@@ -5464,17 +5464,17 @@
       </c>
       <c r="M83" s="0" t="inlineStr">
         <is>
-          <t>4500000335202608122478222937</t>
+          <t>4500000345202608124445297817</t>
         </is>
       </c>
     </row>
     <row r="84" spans="1:14">
       <c r="A84" s="0">
-        <v>49155203</v>
+        <v>49155253</v>
       </c>
       <c r="B84" s="0" t="inlineStr">
         <is>
-          <t>一生有你</t>
+          <t>一顺百顺。好运来</t>
         </is>
       </c>
       <c r="C84" s="0" t="inlineStr">
@@ -5499,7 +5499,7 @@
       </c>
       <c r="G84" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:32:56</t>
+          <t>2026-08-12 21:33:51</t>
         </is>
       </c>
       <c r="H84" s="0" t="inlineStr">
@@ -5529,17 +5529,17 @@
       </c>
       <c r="M84" s="0" t="inlineStr">
         <is>
-          <t>4500000369202608129324316511</t>
+          <t>4500000326202608122909608257</t>
         </is>
       </c>
     </row>
     <row r="85" spans="1:14">
       <c r="A85" s="0">
-        <v>49155200</v>
+        <v>49155246</v>
       </c>
       <c r="B85" s="0" t="inlineStr">
         <is>
-          <t>618</t>
+          <t>陈桂芳</t>
         </is>
       </c>
       <c r="C85" s="0" t="inlineStr">
@@ -5564,7 +5564,7 @@
       </c>
       <c r="G85" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:33:09</t>
+          <t>2026-08-12 21:33:14</t>
         </is>
       </c>
       <c r="H85" s="0" t="inlineStr">
@@ -5594,17 +5594,17 @@
       </c>
       <c r="M85" s="0" t="inlineStr">
         <is>
-          <t>4500000384202608125850014769</t>
+          <t>4500000378202608126828589764</t>
         </is>
       </c>
     </row>
     <row r="86" spans="1:14">
       <c r="A86" s="0">
-        <v>49155197</v>
+        <v>49155234</v>
       </c>
       <c r="B86" s="0" t="inlineStr">
         <is>
-          <t>桂芝改名叫张淑玮</t>
+          <t>黄仲芬15683592716</t>
         </is>
       </c>
       <c r="C86" s="0" t="inlineStr">
@@ -5629,7 +5629,7 @@
       </c>
       <c r="G86" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:33:00</t>
+          <t>2026-08-12 21:33:02</t>
         </is>
       </c>
       <c r="H86" s="0" t="inlineStr">
@@ -5659,17 +5659,17 @@
       </c>
       <c r="M86" s="0" t="inlineStr">
         <is>
-          <t>4500000351202608121228274851</t>
+          <t>4500000325202608129237945248</t>
         </is>
       </c>
     </row>
     <row r="87" spans="1:14">
       <c r="A87" s="0">
-        <v>49155194</v>
+        <v>49155233</v>
       </c>
       <c r="B87" s="0" t="inlineStr">
         <is>
-          <t>自强不息</t>
+          <t>幸福姐赵会玲</t>
         </is>
       </c>
       <c r="C87" s="0" t="inlineStr">
@@ -5694,7 +5694,7 @@
       </c>
       <c r="G87" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:33:14</t>
+          <t>2026-08-12 21:34:04</t>
         </is>
       </c>
       <c r="H87" s="0" t="inlineStr">
@@ -5724,17 +5724,17 @@
       </c>
       <c r="M87" s="0" t="inlineStr">
         <is>
-          <t>4500000356202608124140031616</t>
+          <t>4500000317202608128379976752</t>
         </is>
       </c>
     </row>
     <row r="88" spans="1:14">
       <c r="A88" s="0">
-        <v>49155192</v>
+        <v>49155230</v>
       </c>
       <c r="B88" s="0" t="inlineStr">
         <is>
-          <t>时光如水</t>
+          <t>锦鲤果果</t>
         </is>
       </c>
       <c r="C88" s="0" t="inlineStr">
@@ -5759,7 +5759,7 @@
       </c>
       <c r="G88" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:33:03</t>
+          <t>2026-08-12 21:33:20</t>
         </is>
       </c>
       <c r="H88" s="0" t="inlineStr">
@@ -5789,17 +5789,17 @@
       </c>
       <c r="M88" s="0" t="inlineStr">
         <is>
-          <t>4500000364202608128865933230</t>
+          <t>4500000322202608129199323858</t>
         </is>
       </c>
     </row>
     <row r="89" spans="1:14">
       <c r="A89" s="0">
-        <v>49155187</v>
+        <v>49155226</v>
       </c>
       <c r="B89" s="0" t="inlineStr">
         <is>
-          <t>张丽</t>
+          <t>戎戎</t>
         </is>
       </c>
       <c r="C89" s="0" t="inlineStr">
@@ -5824,7 +5824,7 @@
       </c>
       <c r="G89" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:32:54</t>
+          <t>2026-08-12 21:33:05</t>
         </is>
       </c>
       <c r="H89" s="0" t="inlineStr">
@@ -5854,17 +5854,17 @@
       </c>
       <c r="M89" s="0" t="inlineStr">
         <is>
-          <t>4500000334202608125275144248</t>
+          <t>4500000331202608125827170254</t>
         </is>
       </c>
     </row>
     <row r="90" spans="1:14">
       <c r="A90" s="0">
-        <v>49155186</v>
+        <v>49155220</v>
       </c>
       <c r="B90" s="0" t="inlineStr">
         <is>
-          <t>星辰</t>
+          <t>阿玉</t>
         </is>
       </c>
       <c r="C90" s="0" t="inlineStr">
@@ -5889,7 +5889,7 @@
       </c>
       <c r="G90" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:32:52</t>
+          <t>2026-08-12 21:33:16</t>
         </is>
       </c>
       <c r="H90" s="0" t="inlineStr">
@@ -5919,17 +5919,17 @@
       </c>
       <c r="M90" s="0" t="inlineStr">
         <is>
-          <t>4500000373202608121378976306</t>
+          <t>4500000345202608129272259118</t>
         </is>
       </c>
     </row>
     <row r="91" spans="1:14">
       <c r="A91" s="0">
-        <v>49155185</v>
+        <v>49155219</v>
       </c>
       <c r="B91" s="0" t="inlineStr">
         <is>
-          <t>天津温室大棚光伏厂家18920981728</t>
+          <t>沉淀、</t>
         </is>
       </c>
       <c r="C91" s="0" t="inlineStr">
@@ -5954,7 +5954,7 @@
       </c>
       <c r="G91" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:33:32</t>
+          <t>2026-08-12 21:32:56</t>
         </is>
       </c>
       <c r="H91" s="0" t="inlineStr">
@@ -5984,17 +5984,17 @@
       </c>
       <c r="M91" s="0" t="inlineStr">
         <is>
-          <t>4500000318202608125631581660</t>
+          <t>4500000372202608124305947387</t>
         </is>
       </c>
     </row>
     <row r="92" spans="1:14">
       <c r="A92" s="0">
-        <v>49155184</v>
+        <v>49155216</v>
       </c>
       <c r="B92" s="0" t="inlineStr">
         <is>
-          <t>惠民</t>
+          <t>晴天</t>
         </is>
       </c>
       <c r="C92" s="0" t="inlineStr">
@@ -6019,7 +6019,7 @@
       </c>
       <c r="G92" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:33:08</t>
+          <t>2026-08-12 21:33:07</t>
         </is>
       </c>
       <c r="H92" s="0" t="inlineStr">
@@ -6049,17 +6049,17 @@
       </c>
       <c r="M92" s="0" t="inlineStr">
         <is>
-          <t>4500000355202608121279528970</t>
+          <t>4500000334202608122833385690</t>
         </is>
       </c>
     </row>
     <row r="93" spans="1:14">
       <c r="A93" s="0">
-        <v>49155180</v>
+        <v>49155210</v>
       </c>
       <c r="B93" s="0" t="inlineStr">
         <is>
-          <t>常青树</t>
+          <t>开正商行</t>
         </is>
       </c>
       <c r="C93" s="0" t="inlineStr">
@@ -6084,7 +6084,7 @@
       </c>
       <c r="G93" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:33:06</t>
+          <t>2026-08-12 21:33:02</t>
         </is>
       </c>
       <c r="H93" s="0" t="inlineStr">
@@ -6114,17 +6114,17 @@
       </c>
       <c r="M93" s="0" t="inlineStr">
         <is>
-          <t>4500000357202608125426925788</t>
+          <t>4500000348202608127466098812</t>
         </is>
       </c>
     </row>
     <row r="94" spans="1:14">
       <c r="A94" s="0">
-        <v>49155178</v>
+        <v>49155208</v>
       </c>
       <c r="B94" s="0" t="inlineStr">
         <is>
-          <t>玉伟</t>
+          <t>傻傻的幸福</t>
         </is>
       </c>
       <c r="C94" s="0" t="inlineStr">
@@ -6149,7 +6149,7 @@
       </c>
       <c r="G94" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:33:07</t>
+          <t>2026-08-12 21:32:54</t>
         </is>
       </c>
       <c r="H94" s="0" t="inlineStr">
@@ -6179,17 +6179,17 @@
       </c>
       <c r="M94" s="0" t="inlineStr">
         <is>
-          <t>4500000364202608125205677586</t>
+          <t>4500000378202608122593720010</t>
         </is>
       </c>
     </row>
     <row r="95" spans="1:14">
       <c r="A95" s="0">
-        <v>49155171</v>
+        <v>49155205</v>
       </c>
       <c r="B95" s="0" t="inlineStr">
         <is>
-          <t>秦晓娟～中医五官排毒</t>
+          <t>你好</t>
         </is>
       </c>
       <c r="C95" s="0" t="inlineStr">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="G95" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:33:02</t>
+          <t>2026-08-12 21:32:59</t>
         </is>
       </c>
       <c r="H95" s="0" t="inlineStr">
@@ -6244,17 +6244,17 @@
       </c>
       <c r="M95" s="0" t="inlineStr">
         <is>
-          <t>4500000365202608129265074581</t>
+          <t>4500000335202608122478222937</t>
         </is>
       </c>
     </row>
     <row r="96" spans="1:14">
       <c r="A96" s="0">
-        <v>49155167</v>
+        <v>49155203</v>
       </c>
       <c r="B96" s="0" t="inlineStr">
         <is>
-          <t>水琴</t>
+          <t>一生有你</t>
         </is>
       </c>
       <c r="C96" s="0" t="inlineStr">
@@ -6279,7 +6279,7 @@
       </c>
       <c r="G96" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:32:54</t>
+          <t>2026-08-12 21:32:56</t>
         </is>
       </c>
       <c r="H96" s="0" t="inlineStr">
@@ -6309,17 +6309,17 @@
       </c>
       <c r="M96" s="0" t="inlineStr">
         <is>
-          <t>4500000315202608128554791016</t>
+          <t>4500000369202608129324316511</t>
         </is>
       </c>
     </row>
     <row r="97" spans="1:14">
       <c r="A97" s="0">
-        <v>49155163</v>
+        <v>49155200</v>
       </c>
       <c r="B97" s="0" t="inlineStr">
         <is>
-          <t>祥云ಠ_ಠ</t>
+          <t>618</t>
         </is>
       </c>
       <c r="C97" s="0" t="inlineStr">
@@ -6344,7 +6344,7 @@
       </c>
       <c r="G97" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:32:56</t>
+          <t>2026-08-12 21:33:09</t>
         </is>
       </c>
       <c r="H97" s="0" t="inlineStr">
@@ -6374,17 +6374,17 @@
       </c>
       <c r="M97" s="0" t="inlineStr">
         <is>
-          <t>4500000344202608126804876906</t>
+          <t>4500000384202608125850014769</t>
         </is>
       </c>
     </row>
     <row r="98" spans="1:14">
       <c r="A98" s="0">
-        <v>49155162</v>
+        <v>49155197</v>
       </c>
       <c r="B98" s="0" t="inlineStr">
         <is>
-          <t>雪绒花</t>
+          <t>桂芝改名叫张淑玮</t>
         </is>
       </c>
       <c r="C98" s="0" t="inlineStr">
@@ -6439,17 +6439,17 @@
       </c>
       <c r="M98" s="0" t="inlineStr">
         <is>
-          <t>4500000343202608122943306781</t>
+          <t>4500000351202608121228274851</t>
         </is>
       </c>
     </row>
     <row r="99" spans="1:14">
       <c r="A99" s="0">
-        <v>49155161</v>
+        <v>49155194</v>
       </c>
       <c r="B99" s="0" t="inlineStr">
         <is>
-          <t>        糖果</t>
+          <t>自强不息</t>
         </is>
       </c>
       <c r="C99" s="0" t="inlineStr">
@@ -6474,7 +6474,7 @@
       </c>
       <c r="G99" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:32:52</t>
+          <t>2026-08-12 21:33:14</t>
         </is>
       </c>
       <c r="H99" s="0" t="inlineStr">
@@ -6504,17 +6504,17 @@
       </c>
       <c r="M99" s="0" t="inlineStr">
         <is>
-          <t>4500000384202608121712400624</t>
+          <t>4500000356202608124140031616</t>
         </is>
       </c>
     </row>
     <row r="100" spans="1:14">
       <c r="A100" s="0">
-        <v>49155157</v>
+        <v>49155192</v>
       </c>
       <c r="B100" s="0" t="inlineStr">
         <is>
-          <t>流失的岁月</t>
+          <t>时光如水</t>
         </is>
       </c>
       <c r="C100" s="0" t="inlineStr">
@@ -6539,7 +6539,7 @@
       </c>
       <c r="G100" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:33:11</t>
+          <t>2026-08-12 21:33:03</t>
         </is>
       </c>
       <c r="H100" s="0" t="inlineStr">
@@ -6569,17 +6569,17 @@
       </c>
       <c r="M100" s="0" t="inlineStr">
         <is>
-          <t>4500000379202608126379751055</t>
+          <t>4500000364202608128865933230</t>
         </is>
       </c>
     </row>
     <row r="101" spans="1:14">
       <c r="A101" s="0">
-        <v>49155152</v>
+        <v>49155187</v>
       </c>
       <c r="B101" s="0" t="inlineStr">
         <is>
-          <t>夏末幽荷</t>
+          <t>张丽</t>
         </is>
       </c>
       <c r="C101" s="0" t="inlineStr">
@@ -6604,7 +6604,7 @@
       </c>
       <c r="G101" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:32:49</t>
+          <t>2026-08-12 21:32:54</t>
         </is>
       </c>
       <c r="H101" s="0" t="inlineStr">
@@ -6634,17 +6634,17 @@
       </c>
       <c r="M101" s="0" t="inlineStr">
         <is>
-          <t>4500000337202608128669470764</t>
+          <t>4500000334202608125275144248</t>
         </is>
       </c>
     </row>
     <row r="102" spans="1:14">
       <c r="A102" s="0">
-        <v>49155150</v>
+        <v>49155186</v>
       </c>
       <c r="B102" s="0" t="inlineStr">
         <is>
-          <t>药曼</t>
+          <t>星辰</t>
         </is>
       </c>
       <c r="C102" s="0" t="inlineStr">
@@ -6669,7 +6669,7 @@
       </c>
       <c r="G102" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:32:50</t>
+          <t>2026-08-12 21:32:52</t>
         </is>
       </c>
       <c r="H102" s="0" t="inlineStr">
@@ -6699,17 +6699,17 @@
       </c>
       <c r="M102" s="0" t="inlineStr">
         <is>
-          <t>4500000345202608127294126669</t>
+          <t>4500000373202608121378976306</t>
         </is>
       </c>
     </row>
     <row r="103" spans="1:14">
       <c r="A103" s="0">
-        <v>49155149</v>
+        <v>49155185</v>
       </c>
       <c r="B103" s="0" t="inlineStr">
         <is>
-          <t>🌺 谭谭🌺</t>
+          <t>天津温室大棚光伏厂家18920981728</t>
         </is>
       </c>
       <c r="C103" s="0" t="inlineStr">
@@ -6734,7 +6734,7 @@
       </c>
       <c r="G103" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:32:58</t>
+          <t>2026-08-12 21:33:32</t>
         </is>
       </c>
       <c r="H103" s="0" t="inlineStr">
@@ -6764,17 +6764,17 @@
       </c>
       <c r="M103" s="0" t="inlineStr">
         <is>
-          <t>4500000350202608121029117778</t>
+          <t>4500000318202608125631581660</t>
         </is>
       </c>
     </row>
     <row r="104" spans="1:14">
       <c r="A104" s="0">
-        <v>49155148</v>
+        <v>49155184</v>
       </c>
       <c r="B104" s="0" t="inlineStr">
         <is>
-          <t>王玉(邮局对面卖手机)</t>
+          <t>惠民</t>
         </is>
       </c>
       <c r="C104" s="0" t="inlineStr">
@@ -6799,7 +6799,7 @@
       </c>
       <c r="G104" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:32:49</t>
+          <t>2026-08-12 21:33:08</t>
         </is>
       </c>
       <c r="H104" s="0" t="inlineStr">
@@ -6829,17 +6829,17 @@
       </c>
       <c r="M104" s="0" t="inlineStr">
         <is>
-          <t>4500000342202608126218721690</t>
+          <t>4500000355202608121279528970</t>
         </is>
       </c>
     </row>
     <row r="105" spans="1:14">
       <c r="A105" s="0">
-        <v>49155147</v>
+        <v>49155180</v>
       </c>
       <c r="B105" s="0" t="inlineStr">
         <is>
-          <t>美好夕阳</t>
+          <t>常青树</t>
         </is>
       </c>
       <c r="C105" s="0" t="inlineStr">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="G105" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:32:50</t>
+          <t>2026-08-12 21:33:06</t>
         </is>
       </c>
       <c r="H105" s="0" t="inlineStr">
@@ -6894,17 +6894,17 @@
       </c>
       <c r="M105" s="0" t="inlineStr">
         <is>
-          <t>4500000343202608128224202725</t>
+          <t>4500000357202608125426925788</t>
         </is>
       </c>
     </row>
     <row r="106" spans="1:14">
       <c r="A106" s="0">
-        <v>49155145</v>
+        <v>49155178</v>
       </c>
       <c r="B106" s="0" t="inlineStr">
         <is>
-          <t>平凡</t>
+          <t>玉伟</t>
         </is>
       </c>
       <c r="C106" s="0" t="inlineStr">
@@ -6929,7 +6929,7 @@
       </c>
       <c r="G106" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:32:57</t>
+          <t>2026-08-12 21:33:07</t>
         </is>
       </c>
       <c r="H106" s="0" t="inlineStr">
@@ -6959,17 +6959,17 @@
       </c>
       <c r="M106" s="0" t="inlineStr">
         <is>
-          <t>4500000359202608122476247171</t>
+          <t>4500000364202608125205677586</t>
         </is>
       </c>
     </row>
     <row r="107" spans="1:14">
       <c r="A107" s="0">
-        <v>49155143</v>
+        <v>49155171</v>
       </c>
       <c r="B107" s="0" t="inlineStr">
         <is>
-          <t>唐洪</t>
+          <t>秦晓娟～中医五官排毒</t>
         </is>
       </c>
       <c r="C107" s="0" t="inlineStr">
@@ -6994,7 +6994,7 @@
       </c>
       <c r="G107" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:32:45</t>
+          <t>2026-08-12 21:33:02</t>
         </is>
       </c>
       <c r="H107" s="0" t="inlineStr">
@@ -7024,17 +7024,17 @@
       </c>
       <c r="M107" s="0" t="inlineStr">
         <is>
-          <t>4500000350202608125309483592</t>
+          <t>4500000365202608129265074581</t>
         </is>
       </c>
     </row>
     <row r="108" spans="1:14">
       <c r="A108" s="0">
-        <v>49155140</v>
+        <v>49155167</v>
       </c>
       <c r="B108" s="0" t="inlineStr">
         <is>
-          <t>浅笑</t>
+          <t>水琴</t>
         </is>
       </c>
       <c r="C108" s="0" t="inlineStr">
@@ -7059,7 +7059,7 @@
       </c>
       <c r="G108" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:32:57</t>
+          <t>2026-08-12 21:32:54</t>
         </is>
       </c>
       <c r="H108" s="0" t="inlineStr">
@@ -7089,17 +7089,17 @@
       </c>
       <c r="M108" s="0" t="inlineStr">
         <is>
-          <t>4500000360202608123442658613</t>
+          <t>4500000315202608128554791016</t>
         </is>
       </c>
     </row>
     <row r="109" spans="1:14">
       <c r="A109" s="0">
-        <v>49155137</v>
+        <v>49155163</v>
       </c>
       <c r="B109" s="0" t="inlineStr">
         <is>
-          <t>梅放芳香</t>
+          <t>祥云ಠ_ಠ</t>
         </is>
       </c>
       <c r="C109" s="0" t="inlineStr">
@@ -7124,7 +7124,7 @@
       </c>
       <c r="G109" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:32:59</t>
+          <t>2026-08-12 21:32:56</t>
         </is>
       </c>
       <c r="H109" s="0" t="inlineStr">
@@ -7154,17 +7154,17 @@
       </c>
       <c r="M109" s="0" t="inlineStr">
         <is>
-          <t>4500000356202608127843962862</t>
+          <t>4500000344202608126804876906</t>
         </is>
       </c>
     </row>
     <row r="110" spans="1:14">
       <c r="A110" s="0">
-        <v>49155135</v>
+        <v>49155162</v>
       </c>
       <c r="B110" s="0" t="inlineStr">
         <is>
-          <t>吴素华</t>
+          <t>雪绒花</t>
         </is>
       </c>
       <c r="C110" s="0" t="inlineStr">
@@ -7189,7 +7189,7 @@
       </c>
       <c r="G110" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:32:49</t>
+          <t>2026-08-12 21:33:00</t>
         </is>
       </c>
       <c r="H110" s="0" t="inlineStr">
@@ -7219,17 +7219,17 @@
       </c>
       <c r="M110" s="0" t="inlineStr">
         <is>
-          <t>4500000339202608124292727044</t>
+          <t>4500000343202608122943306781</t>
         </is>
       </c>
     </row>
     <row r="111" spans="1:14">
       <c r="A111" s="0">
-        <v>49155132</v>
+        <v>49155161</v>
       </c>
       <c r="B111" s="0" t="inlineStr">
         <is>
-          <t>苗斯妤铂金牌月嫂催乳18839028160</t>
+          <t>        糖果</t>
         </is>
       </c>
       <c r="C111" s="0" t="inlineStr">
@@ -7254,7 +7254,7 @@
       </c>
       <c r="G111" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:32:46</t>
+          <t>2026-08-12 21:32:52</t>
         </is>
       </c>
       <c r="H111" s="0" t="inlineStr">
@@ -7284,17 +7284,17 @@
       </c>
       <c r="M111" s="0" t="inlineStr">
         <is>
-          <t>4500000322202608123141162109</t>
+          <t>4500000384202608121712400624</t>
         </is>
       </c>
     </row>
     <row r="112" spans="1:14">
       <c r="A112" s="0">
-        <v>49155131</v>
+        <v>49155157</v>
       </c>
       <c r="B112" s="0" t="inlineStr">
         <is>
-          <t>瓷星.</t>
+          <t>流失的岁月</t>
         </is>
       </c>
       <c r="C112" s="0" t="inlineStr">
@@ -7319,7 +7319,7 @@
       </c>
       <c r="G112" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:32:50</t>
+          <t>2026-08-12 21:33:11</t>
         </is>
       </c>
       <c r="H112" s="0" t="inlineStr">
@@ -7349,17 +7349,17 @@
       </c>
       <c r="M112" s="0" t="inlineStr">
         <is>
-          <t>4500000383202608121548709297</t>
+          <t>4500000379202608126379751055</t>
         </is>
       </c>
     </row>
     <row r="113" spans="1:14">
       <c r="A113" s="0">
-        <v>49155129</v>
+        <v>49155152</v>
       </c>
       <c r="B113" s="0" t="inlineStr">
         <is>
-          <t>妈咪宝贝</t>
+          <t>夏末幽荷</t>
         </is>
       </c>
       <c r="C113" s="0" t="inlineStr">
@@ -7384,7 +7384,7 @@
       </c>
       <c r="G113" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:32:42</t>
+          <t>2026-08-12 21:32:49</t>
         </is>
       </c>
       <c r="H113" s="0" t="inlineStr">
@@ -7414,17 +7414,17 @@
       </c>
       <c r="M113" s="0" t="inlineStr">
         <is>
-          <t>4500000347202608127726342481</t>
+          <t>4500000337202608128669470764</t>
         </is>
       </c>
     </row>
     <row r="114" spans="1:14">
       <c r="A114" s="0">
-        <v>49155128</v>
+        <v>49155150</v>
       </c>
       <c r="B114" s="0" t="inlineStr">
         <is>
-          <t>愿结天下有缘人</t>
+          <t>药曼</t>
         </is>
       </c>
       <c r="C114" s="0" t="inlineStr">
@@ -7449,7 +7449,7 @@
       </c>
       <c r="G114" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:32:46</t>
+          <t>2026-08-12 21:32:50</t>
         </is>
       </c>
       <c r="H114" s="0" t="inlineStr">
@@ -7479,17 +7479,17 @@
       </c>
       <c r="M114" s="0" t="inlineStr">
         <is>
-          <t>4500000321202608128699617090</t>
+          <t>4500000345202608127294126669</t>
         </is>
       </c>
     </row>
     <row r="115" spans="1:14">
       <c r="A115" s="0">
-        <v>49155124</v>
+        <v>49155149</v>
       </c>
       <c r="B115" s="0" t="inlineStr">
         <is>
-          <t>勿忘初心</t>
+          <t>🌺 谭谭🌺</t>
         </is>
       </c>
       <c r="C115" s="0" t="inlineStr">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="G115" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:32:49</t>
+          <t>2026-08-12 21:32:58</t>
         </is>
       </c>
       <c r="H115" s="0" t="inlineStr">
@@ -7544,17 +7544,17 @@
       </c>
       <c r="M115" s="0" t="inlineStr">
         <is>
-          <t>4500000373202608128217629837</t>
+          <t>4500000350202608121029117778</t>
         </is>
       </c>
     </row>
     <row r="116" spans="1:14">
       <c r="A116" s="0">
-        <v>49155123</v>
+        <v>49155148</v>
       </c>
       <c r="B116" s="0" t="inlineStr">
         <is>
-          <t>芳草天涯</t>
+          <t>王玉(邮局对面卖手机)</t>
         </is>
       </c>
       <c r="C116" s="0" t="inlineStr">
@@ -7579,7 +7579,7 @@
       </c>
       <c r="G116" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:32:32</t>
+          <t>2026-08-12 21:32:49</t>
         </is>
       </c>
       <c r="H116" s="0" t="inlineStr">
@@ -7609,22 +7609,17 @@
       </c>
       <c r="M116" s="0" t="inlineStr">
         <is>
-          <t>4500000321202608123653997556</t>
-        </is>
-      </c>
-      <c r="N116" s="0" t="inlineStr">
-        <is>
-          <t>合肥</t>
+          <t>4500000342202608126218721690</t>
         </is>
       </c>
     </row>
     <row r="117" spans="1:14">
       <c r="A117" s="0">
-        <v>49155120</v>
+        <v>49155147</v>
       </c>
       <c r="B117" s="0" t="inlineStr">
         <is>
-          <t>记忆中的你</t>
+          <t>美好夕阳</t>
         </is>
       </c>
       <c r="C117" s="0" t="inlineStr">
@@ -7649,7 +7644,7 @@
       </c>
       <c r="G117" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:32:53</t>
+          <t>2026-08-12 21:32:50</t>
         </is>
       </c>
       <c r="H117" s="0" t="inlineStr">
@@ -7679,17 +7674,17 @@
       </c>
       <c r="M117" s="0" t="inlineStr">
         <is>
-          <t>4500000326202608124401684219</t>
+          <t>4500000343202608128224202725</t>
         </is>
       </c>
     </row>
     <row r="118" spans="1:14">
       <c r="A118" s="0">
-        <v>49155114</v>
+        <v>49155145</v>
       </c>
       <c r="B118" s="0" t="inlineStr">
         <is>
-          <t>微笑取暖</t>
+          <t>平凡</t>
         </is>
       </c>
       <c r="C118" s="0" t="inlineStr">
@@ -7714,7 +7709,7 @@
       </c>
       <c r="G118" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:33:38</t>
+          <t>2026-08-12 21:32:57</t>
         </is>
       </c>
       <c r="H118" s="0" t="inlineStr">
@@ -7744,17 +7739,17 @@
       </c>
       <c r="M118" s="0" t="inlineStr">
         <is>
-          <t>4500000325202608121874803628</t>
+          <t>4500000359202608122476247171</t>
         </is>
       </c>
     </row>
     <row r="119" spans="1:14">
       <c r="A119" s="0">
-        <v>49155112</v>
+        <v>49155143</v>
       </c>
       <c r="B119" s="0" t="inlineStr">
         <is>
-          <t>净心李芸</t>
+          <t>唐洪</t>
         </is>
       </c>
       <c r="C119" s="0" t="inlineStr">
@@ -7779,7 +7774,7 @@
       </c>
       <c r="G119" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:32:33</t>
+          <t>2026-08-12 21:32:45</t>
         </is>
       </c>
       <c r="H119" s="0" t="inlineStr">
@@ -7809,17 +7804,17 @@
       </c>
       <c r="M119" s="0" t="inlineStr">
         <is>
-          <t>4500000351202608126115898528</t>
+          <t>4500000350202608125309483592</t>
         </is>
       </c>
     </row>
     <row r="120" spans="1:14">
       <c r="A120" s="0">
-        <v>49155108</v>
+        <v>49155140</v>
       </c>
       <c r="B120" s="0" t="inlineStr">
         <is>
-          <t>衡澜</t>
+          <t>浅笑</t>
         </is>
       </c>
       <c r="C120" s="0" t="inlineStr">
@@ -7844,7 +7839,7 @@
       </c>
       <c r="G120" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:32:32</t>
+          <t>2026-08-12 21:32:57</t>
         </is>
       </c>
       <c r="H120" s="0" t="inlineStr">
@@ -7874,17 +7869,17 @@
       </c>
       <c r="M120" s="0" t="inlineStr">
         <is>
-          <t>4500000360202608128833814214</t>
+          <t>4500000360202608123442658613</t>
         </is>
       </c>
     </row>
     <row r="121" spans="1:14">
       <c r="A121" s="0">
-        <v>49155098</v>
+        <v>49155137</v>
       </c>
       <c r="B121" s="0" t="inlineStr">
         <is>
-          <t>珂</t>
+          <t>梅放芳香</t>
         </is>
       </c>
       <c r="C121" s="0" t="inlineStr">
@@ -7909,7 +7904,7 @@
       </c>
       <c r="G121" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:32:39</t>
+          <t>2026-08-12 21:32:59</t>
         </is>
       </c>
       <c r="H121" s="0" t="inlineStr">
@@ -7939,17 +7934,17 @@
       </c>
       <c r="M121" s="0" t="inlineStr">
         <is>
-          <t>4500000344202608128766183266</t>
+          <t>4500000356202608127843962862</t>
         </is>
       </c>
     </row>
     <row r="122" spans="1:14">
       <c r="A122" s="0">
-        <v>49155095</v>
+        <v>49155135</v>
       </c>
       <c r="B122" s="0" t="inlineStr">
         <is>
-          <t>平安保险~王家宝</t>
+          <t>吴素华</t>
         </is>
       </c>
       <c r="C122" s="0" t="inlineStr">
@@ -7974,7 +7969,7 @@
       </c>
       <c r="G122" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:32:54</t>
+          <t>2026-08-12 21:32:49</t>
         </is>
       </c>
       <c r="H122" s="0" t="inlineStr">
@@ -8004,17 +7999,17 @@
       </c>
       <c r="M122" s="0" t="inlineStr">
         <is>
-          <t>4500000321202608129139460754</t>
+          <t>4500000339202608124292727044</t>
         </is>
       </c>
     </row>
     <row r="123" spans="1:14">
       <c r="A123" s="0">
-        <v>49155092</v>
+        <v>49155132</v>
       </c>
       <c r="B123" s="0" t="inlineStr">
         <is>
-          <t>爱情海</t>
+          <t>苗斯妤铂金牌月嫂催乳18839028160</t>
         </is>
       </c>
       <c r="C123" s="0" t="inlineStr">
@@ -8039,7 +8034,7 @@
       </c>
       <c r="G123" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:32:23</t>
+          <t>2026-08-12 21:32:46</t>
         </is>
       </c>
       <c r="H123" s="0" t="inlineStr">
@@ -8069,17 +8064,17 @@
       </c>
       <c r="M123" s="0" t="inlineStr">
         <is>
-          <t>4500000357202608125918396999</t>
+          <t>4500000322202608123141162109</t>
         </is>
       </c>
     </row>
     <row r="124" spans="1:14">
       <c r="A124" s="0">
-        <v>49155090</v>
+        <v>49155131</v>
       </c>
       <c r="B124" s="0" t="inlineStr">
         <is>
-          <t>三月桃花</t>
+          <t>瓷星.</t>
         </is>
       </c>
       <c r="C124" s="0" t="inlineStr">
@@ -8104,7 +8099,7 @@
       </c>
       <c r="G124" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12 21:32:26</t>
+          <t>2026-08-12 21:32:50</t>
         </is>
       </c>
       <c r="H124" s="0" t="inlineStr">
@@ -8134,70 +8129,855 @@
       </c>
       <c r="M124" s="0" t="inlineStr">
         <is>
-          <t>4500000382202608128744277768</t>
+          <t>4500000383202608121548709297</t>
         </is>
       </c>
     </row>
     <row r="125" spans="1:14">
       <c r="A125" s="0">
+        <v>49155129</v>
+      </c>
+      <c r="B125" s="0" t="inlineStr">
+        <is>
+          <t>妈咪宝贝</t>
+        </is>
+      </c>
+      <c r="C125" s="0" t="inlineStr">
+        <is>
+          <t>【升级版】6天健康瑜伽体验营</t>
+        </is>
+      </c>
+      <c r="D125" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E125" s="0" t="inlineStr">
+        <is>
+          <t>￥1</t>
+        </is>
+      </c>
+      <c r="F125" s="0" t="inlineStr">
+        <is>
+          <t>￥1</t>
+        </is>
+      </c>
+      <c r="G125" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12 21:32:42</t>
+        </is>
+      </c>
+      <c r="H125" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I125" s="0" t="inlineStr">
+        <is>
+          <t>彩虹-抖音1元瑜伽</t>
+        </is>
+      </c>
+      <c r="J125" s="0" t="inlineStr">
+        <is>
+          <t>【WY】瑜伽-气血皮肤（1元 · 支付）</t>
+        </is>
+      </c>
+      <c r="K125" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L125" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="M125" s="0" t="inlineStr">
+        <is>
+          <t>4500000347202608127726342481</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" spans="1:14">
+      <c r="A126" s="0">
+        <v>49155128</v>
+      </c>
+      <c r="B126" s="0" t="inlineStr">
+        <is>
+          <t>愿结天下有缘人</t>
+        </is>
+      </c>
+      <c r="C126" s="0" t="inlineStr">
+        <is>
+          <t>【升级版】6天健康瑜伽体验营</t>
+        </is>
+      </c>
+      <c r="D126" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E126" s="0" t="inlineStr">
+        <is>
+          <t>￥1</t>
+        </is>
+      </c>
+      <c r="F126" s="0" t="inlineStr">
+        <is>
+          <t>￥1</t>
+        </is>
+      </c>
+      <c r="G126" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12 21:32:46</t>
+        </is>
+      </c>
+      <c r="H126" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I126" s="0" t="inlineStr">
+        <is>
+          <t>彩虹-抖音1元瑜伽</t>
+        </is>
+      </c>
+      <c r="J126" s="0" t="inlineStr">
+        <is>
+          <t>【WY】瑜伽-气血皮肤（1元 · 支付）</t>
+        </is>
+      </c>
+      <c r="K126" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L126" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="M126" s="0" t="inlineStr">
+        <is>
+          <t>4500000321202608128699617090</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" spans="1:14">
+      <c r="A127" s="0">
+        <v>49155124</v>
+      </c>
+      <c r="B127" s="0" t="inlineStr">
+        <is>
+          <t>勿忘初心</t>
+        </is>
+      </c>
+      <c r="C127" s="0" t="inlineStr">
+        <is>
+          <t>【升级版】6天健康瑜伽体验营</t>
+        </is>
+      </c>
+      <c r="D127" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E127" s="0" t="inlineStr">
+        <is>
+          <t>￥1</t>
+        </is>
+      </c>
+      <c r="F127" s="0" t="inlineStr">
+        <is>
+          <t>￥1</t>
+        </is>
+      </c>
+      <c r="G127" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12 21:32:49</t>
+        </is>
+      </c>
+      <c r="H127" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I127" s="0" t="inlineStr">
+        <is>
+          <t>彩虹-抖音1元瑜伽</t>
+        </is>
+      </c>
+      <c r="J127" s="0" t="inlineStr">
+        <is>
+          <t>【WY】瑜伽-气血皮肤（1元 · 支付）</t>
+        </is>
+      </c>
+      <c r="K127" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L127" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="M127" s="0" t="inlineStr">
+        <is>
+          <t>4500000373202608128217629837</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" spans="1:14">
+      <c r="A128" s="0">
+        <v>49155123</v>
+      </c>
+      <c r="B128" s="0" t="inlineStr">
+        <is>
+          <t>芳草天涯</t>
+        </is>
+      </c>
+      <c r="C128" s="0" t="inlineStr">
+        <is>
+          <t>【升级版】6天健康瑜伽体验营</t>
+        </is>
+      </c>
+      <c r="D128" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E128" s="0" t="inlineStr">
+        <is>
+          <t>￥1</t>
+        </is>
+      </c>
+      <c r="F128" s="0" t="inlineStr">
+        <is>
+          <t>￥1</t>
+        </is>
+      </c>
+      <c r="G128" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12 21:32:32</t>
+        </is>
+      </c>
+      <c r="H128" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I128" s="0" t="inlineStr">
+        <is>
+          <t>彩虹-抖音1元瑜伽</t>
+        </is>
+      </c>
+      <c r="J128" s="0" t="inlineStr">
+        <is>
+          <t>【WY】瑜伽-气血皮肤（1元 · 支付）</t>
+        </is>
+      </c>
+      <c r="K128" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L128" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="M128" s="0" t="inlineStr">
+        <is>
+          <t>4500000321202608123653997556</t>
+        </is>
+      </c>
+      <c r="N128" s="0" t="inlineStr">
+        <is>
+          <t>合肥</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" spans="1:14">
+      <c r="A129" s="0">
+        <v>49155120</v>
+      </c>
+      <c r="B129" s="0" t="inlineStr">
+        <is>
+          <t>记忆中的你</t>
+        </is>
+      </c>
+      <c r="C129" s="0" t="inlineStr">
+        <is>
+          <t>【升级版】6天健康瑜伽体验营</t>
+        </is>
+      </c>
+      <c r="D129" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E129" s="0" t="inlineStr">
+        <is>
+          <t>￥1</t>
+        </is>
+      </c>
+      <c r="F129" s="0" t="inlineStr">
+        <is>
+          <t>￥1</t>
+        </is>
+      </c>
+      <c r="G129" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12 21:32:53</t>
+        </is>
+      </c>
+      <c r="H129" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I129" s="0" t="inlineStr">
+        <is>
+          <t>彩虹-抖音1元瑜伽</t>
+        </is>
+      </c>
+      <c r="J129" s="0" t="inlineStr">
+        <is>
+          <t>【WY】瑜伽-气血皮肤（1元 · 支付）</t>
+        </is>
+      </c>
+      <c r="K129" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L129" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="M129" s="0" t="inlineStr">
+        <is>
+          <t>4500000326202608124401684219</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" spans="1:14">
+      <c r="A130" s="0">
+        <v>49155114</v>
+      </c>
+      <c r="B130" s="0" t="inlineStr">
+        <is>
+          <t>微笑取暖</t>
+        </is>
+      </c>
+      <c r="C130" s="0" t="inlineStr">
+        <is>
+          <t>【升级版】6天健康瑜伽体验营</t>
+        </is>
+      </c>
+      <c r="D130" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E130" s="0" t="inlineStr">
+        <is>
+          <t>￥1</t>
+        </is>
+      </c>
+      <c r="F130" s="0" t="inlineStr">
+        <is>
+          <t>￥1</t>
+        </is>
+      </c>
+      <c r="G130" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12 21:33:38</t>
+        </is>
+      </c>
+      <c r="H130" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I130" s="0" t="inlineStr">
+        <is>
+          <t>彩虹-抖音1元瑜伽</t>
+        </is>
+      </c>
+      <c r="J130" s="0" t="inlineStr">
+        <is>
+          <t>【WY】瑜伽-气血皮肤（1元 · 支付）</t>
+        </is>
+      </c>
+      <c r="K130" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L130" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="M130" s="0" t="inlineStr">
+        <is>
+          <t>4500000325202608121874803628</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" spans="1:14">
+      <c r="A131" s="0">
+        <v>49155112</v>
+      </c>
+      <c r="B131" s="0" t="inlineStr">
+        <is>
+          <t>净心李芸</t>
+        </is>
+      </c>
+      <c r="C131" s="0" t="inlineStr">
+        <is>
+          <t>【升级版】6天健康瑜伽体验营</t>
+        </is>
+      </c>
+      <c r="D131" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E131" s="0" t="inlineStr">
+        <is>
+          <t>￥1</t>
+        </is>
+      </c>
+      <c r="F131" s="0" t="inlineStr">
+        <is>
+          <t>￥1</t>
+        </is>
+      </c>
+      <c r="G131" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12 21:32:33</t>
+        </is>
+      </c>
+      <c r="H131" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I131" s="0" t="inlineStr">
+        <is>
+          <t>彩虹-抖音1元瑜伽</t>
+        </is>
+      </c>
+      <c r="J131" s="0" t="inlineStr">
+        <is>
+          <t>【WY】瑜伽-气血皮肤（1元 · 支付）</t>
+        </is>
+      </c>
+      <c r="K131" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L131" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="M131" s="0" t="inlineStr">
+        <is>
+          <t>4500000351202608126115898528</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" spans="1:14">
+      <c r="A132" s="0">
+        <v>49155108</v>
+      </c>
+      <c r="B132" s="0" t="inlineStr">
+        <is>
+          <t>衡澜</t>
+        </is>
+      </c>
+      <c r="C132" s="0" t="inlineStr">
+        <is>
+          <t>【升级版】6天健康瑜伽体验营</t>
+        </is>
+      </c>
+      <c r="D132" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E132" s="0" t="inlineStr">
+        <is>
+          <t>￥1</t>
+        </is>
+      </c>
+      <c r="F132" s="0" t="inlineStr">
+        <is>
+          <t>￥1</t>
+        </is>
+      </c>
+      <c r="G132" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12 21:32:32</t>
+        </is>
+      </c>
+      <c r="H132" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I132" s="0" t="inlineStr">
+        <is>
+          <t>彩虹-抖音1元瑜伽</t>
+        </is>
+      </c>
+      <c r="J132" s="0" t="inlineStr">
+        <is>
+          <t>【WY】瑜伽-气血皮肤（1元 · 支付）</t>
+        </is>
+      </c>
+      <c r="K132" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L132" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="M132" s="0" t="inlineStr">
+        <is>
+          <t>4500000360202608128833814214</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" spans="1:14">
+      <c r="A133" s="0">
+        <v>49155098</v>
+      </c>
+      <c r="B133" s="0" t="inlineStr">
+        <is>
+          <t>珂</t>
+        </is>
+      </c>
+      <c r="C133" s="0" t="inlineStr">
+        <is>
+          <t>【升级版】6天健康瑜伽体验营</t>
+        </is>
+      </c>
+      <c r="D133" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E133" s="0" t="inlineStr">
+        <is>
+          <t>￥1</t>
+        </is>
+      </c>
+      <c r="F133" s="0" t="inlineStr">
+        <is>
+          <t>￥1</t>
+        </is>
+      </c>
+      <c r="G133" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12 21:32:39</t>
+        </is>
+      </c>
+      <c r="H133" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I133" s="0" t="inlineStr">
+        <is>
+          <t>彩虹-抖音1元瑜伽</t>
+        </is>
+      </c>
+      <c r="J133" s="0" t="inlineStr">
+        <is>
+          <t>【WY】瑜伽-气血皮肤（1元 · 支付）</t>
+        </is>
+      </c>
+      <c r="K133" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L133" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="M133" s="0" t="inlineStr">
+        <is>
+          <t>4500000344202608128766183266</t>
+        </is>
+      </c>
+    </row>
+    <row r="134" spans="1:14">
+      <c r="A134" s="0">
+        <v>49155095</v>
+      </c>
+      <c r="B134" s="0" t="inlineStr">
+        <is>
+          <t>平安保险~王家宝</t>
+        </is>
+      </c>
+      <c r="C134" s="0" t="inlineStr">
+        <is>
+          <t>【升级版】6天健康瑜伽体验营</t>
+        </is>
+      </c>
+      <c r="D134" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E134" s="0" t="inlineStr">
+        <is>
+          <t>￥1</t>
+        </is>
+      </c>
+      <c r="F134" s="0" t="inlineStr">
+        <is>
+          <t>￥1</t>
+        </is>
+      </c>
+      <c r="G134" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12 21:32:54</t>
+        </is>
+      </c>
+      <c r="H134" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I134" s="0" t="inlineStr">
+        <is>
+          <t>彩虹-抖音1元瑜伽</t>
+        </is>
+      </c>
+      <c r="J134" s="0" t="inlineStr">
+        <is>
+          <t>【WY】瑜伽-气血皮肤（1元 · 支付）</t>
+        </is>
+      </c>
+      <c r="K134" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L134" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="M134" s="0" t="inlineStr">
+        <is>
+          <t>4500000321202608129139460754</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" spans="1:14">
+      <c r="A135" s="0">
+        <v>49155092</v>
+      </c>
+      <c r="B135" s="0" t="inlineStr">
+        <is>
+          <t>爱情海</t>
+        </is>
+      </c>
+      <c r="C135" s="0" t="inlineStr">
+        <is>
+          <t>【升级版】6天健康瑜伽体验营</t>
+        </is>
+      </c>
+      <c r="D135" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E135" s="0" t="inlineStr">
+        <is>
+          <t>￥1</t>
+        </is>
+      </c>
+      <c r="F135" s="0" t="inlineStr">
+        <is>
+          <t>￥1</t>
+        </is>
+      </c>
+      <c r="G135" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12 21:32:23</t>
+        </is>
+      </c>
+      <c r="H135" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I135" s="0" t="inlineStr">
+        <is>
+          <t>彩虹-抖音1元瑜伽</t>
+        </is>
+      </c>
+      <c r="J135" s="0" t="inlineStr">
+        <is>
+          <t>【WY】瑜伽-气血皮肤（1元 · 支付）</t>
+        </is>
+      </c>
+      <c r="K135" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L135" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="M135" s="0" t="inlineStr">
+        <is>
+          <t>4500000357202608125918396999</t>
+        </is>
+      </c>
+    </row>
+    <row r="136" spans="1:14">
+      <c r="A136" s="0">
+        <v>49155090</v>
+      </c>
+      <c r="B136" s="0" t="inlineStr">
+        <is>
+          <t>三月桃花</t>
+        </is>
+      </c>
+      <c r="C136" s="0" t="inlineStr">
+        <is>
+          <t>【升级版】6天健康瑜伽体验营</t>
+        </is>
+      </c>
+      <c r="D136" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E136" s="0" t="inlineStr">
+        <is>
+          <t>￥1</t>
+        </is>
+      </c>
+      <c r="F136" s="0" t="inlineStr">
+        <is>
+          <t>￥1</t>
+        </is>
+      </c>
+      <c r="G136" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12 21:32:26</t>
+        </is>
+      </c>
+      <c r="H136" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I136" s="0" t="inlineStr">
+        <is>
+          <t>彩虹-抖音1元瑜伽</t>
+        </is>
+      </c>
+      <c r="J136" s="0" t="inlineStr">
+        <is>
+          <t>【WY】瑜伽-气血皮肤（1元 · 支付）</t>
+        </is>
+      </c>
+      <c r="K136" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L136" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="M136" s="0" t="inlineStr">
+        <is>
+          <t>4500000382202608128744277768</t>
+        </is>
+      </c>
+    </row>
+    <row r="137" spans="1:14">
+      <c r="A137" s="0">
         <v>49155088</v>
       </c>
-      <c r="B125" s="0" t="inlineStr">
+      <c r="B137" s="0" t="inlineStr">
         <is>
           <t>绘兰艺术李老师</t>
         </is>
       </c>
-      <c r="C125" s="0" t="inlineStr">
-        <is>
-          <t>【升级版】6天健康瑜伽体验营</t>
-        </is>
-      </c>
-      <c r="D125" s="0" t="inlineStr">
-        <is>
-          <t>训练营</t>
-        </is>
-      </c>
-      <c r="E125" s="0" t="inlineStr">
-        <is>
-          <t>￥1</t>
-        </is>
-      </c>
-      <c r="F125" s="0" t="inlineStr">
-        <is>
-          <t>￥1</t>
-        </is>
-      </c>
-      <c r="G125" s="0" t="inlineStr">
+      <c r="C137" s="0" t="inlineStr">
+        <is>
+          <t>【升级版】6天健康瑜伽体验营</t>
+        </is>
+      </c>
+      <c r="D137" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E137" s="0" t="inlineStr">
+        <is>
+          <t>￥1</t>
+        </is>
+      </c>
+      <c r="F137" s="0" t="inlineStr">
+        <is>
+          <t>￥1</t>
+        </is>
+      </c>
+      <c r="G137" s="0" t="inlineStr">
         <is>
           <t>2026-08-12 21:32:20</t>
         </is>
       </c>
-      <c r="H125" s="0" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I125" s="0" t="inlineStr">
-        <is>
-          <t>彩虹-抖音1元瑜伽</t>
-        </is>
-      </c>
-      <c r="J125" s="0" t="inlineStr">
-        <is>
-          <t>【WY】瑜伽-气血皮肤（1元 · 支付）</t>
-        </is>
-      </c>
-      <c r="K125" s="0" t="inlineStr">
-        <is>
-          <t>微信支付</t>
-        </is>
-      </c>
-      <c r="L125" s="0" t="inlineStr">
-        <is>
-          <t>已完成</t>
-        </is>
-      </c>
-      <c r="M125" s="0" t="inlineStr">
+      <c r="H137" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I137" s="0" t="inlineStr">
+        <is>
+          <t>彩虹-抖音1元瑜伽</t>
+        </is>
+      </c>
+      <c r="J137" s="0" t="inlineStr">
+        <is>
+          <t>【WY】瑜伽-气血皮肤（1元 · 支付）</t>
+        </is>
+      </c>
+      <c r="K137" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L137" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="M137" s="0" t="inlineStr">
         <is>
           <t>4500000358202608128940402527</t>
         </is>

</xml_diff>